<commit_message>
Se agregó la data de las parroquias a la aplicación
</commit_message>
<xml_diff>
--- a/libro_publicaciones.xlsx
+++ b/libro_publicaciones.xlsx
@@ -5,14 +5,14 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fguedez\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fguedez\Documents\Proyectos\page-estadisticas\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7905"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7905" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="publicaciones" sheetId="2" r:id="rId1"/>
+    <sheet name="data_parroquia" sheetId="2" r:id="rId1"/>
     <sheet name="parr-data" sheetId="3" r:id="rId2"/>
     <sheet name="dpt_delta" sheetId="1" r:id="rId3"/>
     <sheet name="formato" sheetId="4" r:id="rId4"/>
@@ -411,9 +411,6 @@
   </cellStyles>
   <dxfs count="3">
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -449,6 +446,9 @@
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -467,11 +467,11 @@
   <autoFilter ref="A1:F28"/>
   <tableColumns count="6">
     <tableColumn id="1" name="cod_dpt"/>
-    <tableColumn id="2" name="cod_publicacion" dataDxfId="0">
+    <tableColumn id="2" name="cod_publicacion" dataDxfId="2">
       <calculatedColumnFormula>ROW(A1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" name="title" dataDxfId="2"/>
-    <tableColumn id="4" name="descripcion" dataDxfId="1"/>
+    <tableColumn id="3" name="title" dataDxfId="1"/>
+    <tableColumn id="4" name="descripcion" dataDxfId="0"/>
     <tableColumn id="5" name="format"/>
     <tableColumn id="6" name="url" dataCellStyle="Hipervínculo"/>
   </tableColumns>
@@ -841,7 +841,7 @@
         <v>19</v>
       </c>
       <c r="B5" s="4">
-        <f>ROW(A4)</f>
+        <f t="shared" ref="B5:B28" si="1">ROW(A4)</f>
         <v>4</v>
       </c>
       <c r="C5" s="5" t="s">
@@ -862,7 +862,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="4">
-        <f>ROW(A5)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="C6" s="5" t="s">
@@ -883,7 +883,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="4">
-        <f>ROW(A6)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="C7" s="5" t="s">
@@ -904,7 +904,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="4">
-        <f>ROW(A7)</f>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="C8" s="5" t="s">
@@ -925,7 +925,7 @@
         <v>4</v>
       </c>
       <c r="B9" s="4">
-        <f>ROW(A8)</f>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="C9" s="5" t="s">
@@ -946,7 +946,7 @@
         <v>4</v>
       </c>
       <c r="B10" s="4">
-        <f>ROW(A9)</f>
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="C10" s="5" t="s">
@@ -967,7 +967,7 @@
         <v>4</v>
       </c>
       <c r="B11" s="4">
-        <f>ROW(A10)</f>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="C11" s="5" t="s">
@@ -988,7 +988,7 @@
         <v>4</v>
       </c>
       <c r="B12" s="4">
-        <f>ROW(A11)</f>
+        <f t="shared" si="1"/>
         <v>11</v>
       </c>
       <c r="C12" s="5" t="s">
@@ -1009,7 +1009,7 @@
         <v>4</v>
       </c>
       <c r="B13" s="4">
-        <f>ROW(A12)</f>
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="C13" s="5" t="s">
@@ -1030,7 +1030,7 @@
         <v>4</v>
       </c>
       <c r="B14" s="4">
-        <f>ROW(A13)</f>
+        <f t="shared" si="1"/>
         <v>13</v>
       </c>
       <c r="C14" s="5" t="s">
@@ -1051,7 +1051,7 @@
         <v>4</v>
       </c>
       <c r="B15" s="4">
-        <f>ROW(A14)</f>
+        <f t="shared" si="1"/>
         <v>14</v>
       </c>
       <c r="C15" s="5" t="s">
@@ -1072,7 +1072,7 @@
         <v>4</v>
       </c>
       <c r="B16" s="4">
-        <f>ROW(A15)</f>
+        <f t="shared" si="1"/>
         <v>15</v>
       </c>
       <c r="C16" s="5" t="s">
@@ -1093,7 +1093,7 @@
         <v>4</v>
       </c>
       <c r="B17" s="4">
-        <f>ROW(A16)</f>
+        <f t="shared" si="1"/>
         <v>16</v>
       </c>
       <c r="C17" s="5" t="s">
@@ -1114,7 +1114,7 @@
         <v>4</v>
       </c>
       <c r="B18" s="4">
-        <f>ROW(A17)</f>
+        <f t="shared" si="1"/>
         <v>17</v>
       </c>
       <c r="C18" s="5" t="s">
@@ -1135,7 +1135,7 @@
         <v>4</v>
       </c>
       <c r="B19" s="4">
-        <f>ROW(A18)</f>
+        <f t="shared" si="1"/>
         <v>18</v>
       </c>
       <c r="C19" s="5" t="s">
@@ -1156,7 +1156,7 @@
         <v>4</v>
       </c>
       <c r="B20" s="4">
-        <f>ROW(A19)</f>
+        <f t="shared" si="1"/>
         <v>19</v>
       </c>
       <c r="C20" s="5" t="s">
@@ -1177,7 +1177,7 @@
         <v>4</v>
       </c>
       <c r="B21" s="4">
-        <f>ROW(A20)</f>
+        <f t="shared" si="1"/>
         <v>20</v>
       </c>
       <c r="C21" s="5" t="s">
@@ -1198,7 +1198,7 @@
         <v>4</v>
       </c>
       <c r="B22" s="4">
-        <f>ROW(A21)</f>
+        <f t="shared" si="1"/>
         <v>21</v>
       </c>
       <c r="C22" s="5" t="s">
@@ -1219,7 +1219,7 @@
         <v>4</v>
       </c>
       <c r="B23" s="4">
-        <f>ROW(A22)</f>
+        <f t="shared" si="1"/>
         <v>22</v>
       </c>
       <c r="C23" s="5" t="s">
@@ -1240,7 +1240,7 @@
         <v>4</v>
       </c>
       <c r="B24" s="4">
-        <f>ROW(A23)</f>
+        <f t="shared" si="1"/>
         <v>23</v>
       </c>
       <c r="C24" s="5" t="s">
@@ -1261,7 +1261,7 @@
         <v>13</v>
       </c>
       <c r="B25" s="4">
-        <f>ROW(A24)</f>
+        <f t="shared" si="1"/>
         <v>24</v>
       </c>
       <c r="C25" s="5" t="s">
@@ -1282,7 +1282,7 @@
         <v>4</v>
       </c>
       <c r="B26" s="4">
-        <f>ROW(A25)</f>
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
       <c r="C26" s="5" t="s">
@@ -1303,7 +1303,7 @@
         <v>14</v>
       </c>
       <c r="B27" s="4">
-        <f>ROW(A26)</f>
+        <f t="shared" si="1"/>
         <v>26</v>
       </c>
       <c r="C27" s="5" t="s">
@@ -1324,7 +1324,7 @@
         <v>23</v>
       </c>
       <c r="B28" s="4">
-        <f>ROW(A27)</f>
+        <f t="shared" si="1"/>
         <v>27</v>
       </c>
       <c r="C28" s="5" t="s">

</xml_diff>

<commit_message>
Se agregó la parroquia Padre Barral Santos Abelgas
</commit_message>
<xml_diff>
--- a/libro_publicaciones.xlsx
+++ b/libro_publicaciones.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7905" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7905"/>
   </bookViews>
   <sheets>
     <sheet name="data_parroquia" sheetId="2" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="170">
   <si>
     <t>codigo</t>
   </si>
@@ -107,9 +107,6 @@
     <t>cod_dpt</t>
   </si>
   <si>
-    <t>descripcion</t>
-  </si>
-  <si>
     <t>url</t>
   </si>
   <si>
@@ -324,6 +321,222 @@
   </si>
   <si>
     <t>https://docs.google.com/presentation/d/1v354uD4Wq5tUS3q32K-7Tot1dqModJbb/edit?usp=drive_link&amp;ouid=105142876406402750370&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1kiGrAKpKFzvMIas5XiA-nwVBZ6ZCEX25/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/179KUodqofy8urV712zsOityyUree352T/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA Y CENTRO POBLADO BOCA DE ARAGUAO</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA Y CENTRO POBLADO POTRERITO</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA Y CENTRO POBLADO RAMANCE DE SACUPANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1IynOfRXoLoEg__G6RrzANlSGVftxjXaK/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA Y CENTRO JANAMANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1ojy5jD-Wlgcj1OvN_S8soiIRtKX15n9Y/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA Y CENTRO POBLADO BOCA DE SACUPANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1qGHkjsLvHRDloSnfztUOkQaoO2s61akh/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA Y CENTRO POBLADO CUBERINA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1BopfCadXeFKi4oQrPdBS-G4PUZebq55q/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA Y CENTRO POBLADO ISLA EL NORTE</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1Ae_hTO6TSZNgDwwjQNxNcNC7vD5Ca-ZU/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA DAUWARUBAKA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1POB3lReTP17OkPQXqb_rvtL-MdLOYpPK/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA KAMAWI</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1JROglhalrOs6rdsM9nPinHF3VPaf-p3e/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA DAUDAJANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1BF07ztO0hOxsFOKFC0g-YS-q2iCbhgRc/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA JEBUANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1XTKlGG-IyD4qMb2Wu8neENQ_m676IVRI/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA JOKABANOKO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1xQkLEqJkJQIL8RIwmr3feu59I4ycXoNV/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA EKUJANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/189Gm2uiferZC8Rvgu1XTDHiWxZOTjCf-/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA JAJERUINA III</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1g0SyNUpDb0K0DDeFeyc8Fexa_ZPAE54m/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA JOROBADO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1w207E68RPTHJFnmPjeFWzB9HR7_MUqKm/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA MEREJINA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1eqzS58Kfsl6FuTJa2m1MYnQmxD0bznrs/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA MORAJANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1UuSveQmH4NlmuYu1b3FbcfewtyXgykIS/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA ARUWAJABANOKO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1Ckryj7J5iy-G_Cp-RMrZC3epGAgt3qXQ/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA JUANACEBE</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1YxjbeB3zPVm9EkcSuT0VLrL_J8bt9WY8/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA KARIBASA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1_sljahFLvHw8WP-qAiAIOgA_0uYeJbmZ/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA WABIAJEBERENOKO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1zw2F-3h1ZcCXibLp7HESZFKTdTBUJ9a-/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA IKARUINA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1NPWiQxA6vMXCnz4-jLk4fh6foIV9W0-W/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA BUBAKA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1P_XEjN-DIW3TgXhsV4dWpWwgqOb71aIe/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA JOTAJANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1zhuDQZdUFOiaKz05Wl_7YgidscOihjfp/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA COCAL</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/17uLrMoai1JfE3wtPdbro9FXxqn8vykxD/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA NABAWAJA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1WGSK11ChwV8dYi2AQaqSyyxQyeCdfEcW/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA CAIMAN</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1MuvYx7ynILsrmqJ9IrG6bWCG_AtLtF82/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA WARAINA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1k4TXvwvIWZdXYuKsBBGRxbEq80r-OFPq/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA AJOTEJANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/191jOus1mjI8BgBN3vlXXntSSt9nLh6dK/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA DAKOJI</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/12sTb4tkP6yxjXf3xcW2ARaSgKDf-4uDH/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA ASIJANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1FDXIgzMiRqALHugglym6f7ZgU2rWnnaD/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA JAJERUINA </t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1MSrxQFlS_vmDiM842NuG9zYwv9ndxv2E/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA BAKAMU</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1Zix2g8A1YoVaIFIw90NRwHeZnW0qXWdF/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA GUAYABOROINA DE GUAYO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1ewO6R8bs-Cag9OTCb5Ue9hh9lFLW9ky-/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA WANEKO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1IFU6MNtrIOM0VTcV3Fdn84BFDqJ20TCF/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA AIMURUINA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1PzvKm47faiNB3g73QdKmLGO8Uqg6KMr9/view?usp=drive_link</t>
   </si>
 </sst>
 </file>
@@ -463,15 +676,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:F28" totalsRowShown="0">
-  <autoFilter ref="A1:F28"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:F64" totalsRowShown="0">
+  <autoFilter ref="A1:F64"/>
   <tableColumns count="6">
     <tableColumn id="1" name="cod_dpt"/>
     <tableColumn id="2" name="cod_publicacion" dataDxfId="2">
       <calculatedColumnFormula>ROW(A1)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="3" name="title" dataDxfId="1"/>
-    <tableColumn id="4" name="descripcion" dataDxfId="0"/>
+    <tableColumn id="4" name="description" dataDxfId="0"/>
     <tableColumn id="5" name="format"/>
     <tableColumn id="6" name="url" dataCellStyle="Hipervínculo"/>
   </tableColumns>
@@ -742,13 +955,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="21.140625" customWidth="1"/>
-    <col min="3" max="3" width="62.28515625" customWidth="1"/>
-    <col min="4" max="4" width="64.28515625" customWidth="1"/>
+    <col min="3" max="3" width="59.28515625" customWidth="1"/>
+    <col min="4" max="4" width="77.85546875" customWidth="1"/>
     <col min="5" max="5" width="19.28515625" customWidth="1"/>
     <col min="6" max="6" width="34.42578125" customWidth="1"/>
   </cols>
@@ -758,19 +971,19 @@
         <v>25</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" t="s">
         <v>26</v>
-      </c>
-      <c r="E1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F1" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -782,16 +995,16 @@
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -803,16 +1016,16 @@
         <v>2</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="E3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -824,16 +1037,16 @@
         <v>3</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="E4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -845,16 +1058,16 @@
         <v>4</v>
       </c>
       <c r="C5" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E5" t="s">
-        <v>28</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -866,16 +1079,16 @@
         <v>5</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E6" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="E6" t="s">
-        <v>28</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -887,16 +1100,16 @@
         <v>6</v>
       </c>
       <c r="C7" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="E7" t="s">
-        <v>29</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -908,16 +1121,16 @@
         <v>7</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D8" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="E8" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="E8" t="s">
-        <v>29</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -929,16 +1142,16 @@
         <v>8</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D9" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="E9" t="s">
-        <v>29</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -950,16 +1163,16 @@
         <v>9</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D10" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="E10" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="E10" t="s">
-        <v>29</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -971,16 +1184,16 @@
         <v>10</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D11" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="E11" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="E11" t="s">
-        <v>29</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -992,16 +1205,16 @@
         <v>11</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D12" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E12" t="s">
+        <v>28</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="E12" t="s">
-        <v>29</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1013,16 +1226,16 @@
         <v>12</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D13" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="E13" t="s">
-        <v>29</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1034,16 +1247,16 @@
         <v>13</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D14" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="E14" t="s">
+        <v>28</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="E14" t="s">
-        <v>29</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1055,16 +1268,16 @@
         <v>14</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D15" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E15" t="s">
+        <v>28</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="E15" t="s">
-        <v>29</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1076,16 +1289,16 @@
         <v>15</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D16" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E16" t="s">
+        <v>28</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="E16" t="s">
-        <v>29</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1097,16 +1310,16 @@
         <v>16</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D17" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E17" t="s">
+        <v>28</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>77</v>
-      </c>
-      <c r="E17" t="s">
-        <v>29</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -1118,16 +1331,16 @@
         <v>17</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D18" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="E18" t="s">
+        <v>28</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="E18" t="s">
-        <v>29</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1139,16 +1352,16 @@
         <v>18</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D19" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="E19" t="s">
+        <v>28</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="E19" t="s">
-        <v>29</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -1160,16 +1373,16 @@
         <v>19</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D20" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="E20" t="s">
+        <v>28</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>83</v>
-      </c>
-      <c r="E20" t="s">
-        <v>29</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1181,16 +1394,16 @@
         <v>20</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D21" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="E21" t="s">
+        <v>28</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>83</v>
-      </c>
-      <c r="E21" t="s">
-        <v>29</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1202,16 +1415,16 @@
         <v>21</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1223,16 +1436,16 @@
         <v>22</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E23" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -1244,16 +1457,16 @@
         <v>23</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D24" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E24" t="s">
+        <v>28</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="E24" t="s">
-        <v>29</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1265,16 +1478,16 @@
         <v>24</v>
       </c>
       <c r="C25" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E25" t="s">
+        <v>27</v>
+      </c>
+      <c r="F25" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="E25" t="s">
-        <v>28</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -1286,16 +1499,16 @@
         <v>25</v>
       </c>
       <c r="C26" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="D26" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="E26" t="s">
+        <v>27</v>
+      </c>
+      <c r="F26" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="E26" t="s">
-        <v>28</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1307,16 +1520,16 @@
         <v>26</v>
       </c>
       <c r="C27" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="E27" t="s">
+        <v>27</v>
+      </c>
+      <c r="F27" s="1" t="s">
         <v>95</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="E27" t="s">
-        <v>28</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -1328,16 +1541,772 @@
         <v>27</v>
       </c>
       <c r="C28" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="E28" t="s">
+        <v>27</v>
+      </c>
+      <c r="F28" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="D28" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="E28" t="s">
-        <v>28</v>
-      </c>
-      <c r="F28" s="1" t="s">
+    </row>
+    <row r="29" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B29" s="4">
+        <f t="shared" ref="B29:B30" si="2">ROW(A28)</f>
+        <v>28</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="E29" t="s">
+        <v>28</v>
+      </c>
+      <c r="F29" s="1" t="s">
         <v>98</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>8</v>
+      </c>
+      <c r="B30" s="4">
+        <f t="shared" si="2"/>
+        <v>29</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="E30" t="s">
+        <v>28</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>8</v>
+      </c>
+      <c r="B31" s="4">
+        <f t="shared" ref="B31:B32" si="3">ROW(A30)</f>
+        <v>30</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="E31" t="s">
+        <v>28</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>8</v>
+      </c>
+      <c r="B32" s="4">
+        <f t="shared" si="3"/>
+        <v>31</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E32" t="s">
+        <v>28</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>8</v>
+      </c>
+      <c r="B33" s="4">
+        <f t="shared" ref="B33:B34" si="4">ROW(A32)</f>
+        <v>32</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="E33" t="s">
+        <v>28</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>8</v>
+      </c>
+      <c r="B34" s="4">
+        <f t="shared" si="4"/>
+        <v>33</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="E34" t="s">
+        <v>28</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>8</v>
+      </c>
+      <c r="B35" s="4">
+        <f t="shared" ref="B35:B36" si="5">ROW(A34)</f>
+        <v>34</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="E35" t="s">
+        <v>28</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>7</v>
+      </c>
+      <c r="B36" s="4">
+        <f t="shared" si="5"/>
+        <v>35</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="E36" t="s">
+        <v>28</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>7</v>
+      </c>
+      <c r="B37" s="4">
+        <f t="shared" ref="B37:B38" si="6">ROW(A36)</f>
+        <v>36</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="E37" t="s">
+        <v>28</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>7</v>
+      </c>
+      <c r="B38" s="4">
+        <f t="shared" si="6"/>
+        <v>37</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="E38" t="s">
+        <v>28</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>7</v>
+      </c>
+      <c r="B39" s="4">
+        <f t="shared" ref="B39:B40" si="7">ROW(A38)</f>
+        <v>38</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="E39" t="s">
+        <v>28</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>7</v>
+      </c>
+      <c r="B40" s="4">
+        <f t="shared" si="7"/>
+        <v>39</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="E40" t="s">
+        <v>28</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>7</v>
+      </c>
+      <c r="B41" s="4">
+        <f t="shared" ref="B41:B42" si="8">ROW(A40)</f>
+        <v>40</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="E41" t="s">
+        <v>28</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>7</v>
+      </c>
+      <c r="B42" s="4">
+        <f t="shared" si="8"/>
+        <v>41</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="E42" t="s">
+        <v>28</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>7</v>
+      </c>
+      <c r="B43" s="4">
+        <f t="shared" ref="B43:B44" si="9">ROW(A42)</f>
+        <v>42</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="E43" t="s">
+        <v>28</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>7</v>
+      </c>
+      <c r="B44" s="4">
+        <f t="shared" si="9"/>
+        <v>43</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="E44" t="s">
+        <v>28</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>7</v>
+      </c>
+      <c r="B45" s="4">
+        <f t="shared" ref="B45:B46" si="10">ROW(A44)</f>
+        <v>44</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E45" t="s">
+        <v>28</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>7</v>
+      </c>
+      <c r="B46" s="4">
+        <f t="shared" si="10"/>
+        <v>45</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="E46" t="s">
+        <v>28</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>7</v>
+      </c>
+      <c r="B47" s="4">
+        <f t="shared" ref="B47:B48" si="11">ROW(A46)</f>
+        <v>46</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="E47" t="s">
+        <v>28</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>7</v>
+      </c>
+      <c r="B48" s="4">
+        <f t="shared" si="11"/>
+        <v>47</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="E48" t="s">
+        <v>28</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>7</v>
+      </c>
+      <c r="B49" s="4">
+        <f t="shared" ref="B49:B50" si="12">ROW(A48)</f>
+        <v>48</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="E49" t="s">
+        <v>28</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>7</v>
+      </c>
+      <c r="B50" s="4">
+        <f t="shared" si="12"/>
+        <v>49</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="E50" t="s">
+        <v>28</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>7</v>
+      </c>
+      <c r="B51" s="4">
+        <f t="shared" ref="B51:B52" si="13">ROW(A50)</f>
+        <v>50</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="E51" t="s">
+        <v>28</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>7</v>
+      </c>
+      <c r="B52" s="4">
+        <f t="shared" si="13"/>
+        <v>51</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="E52" t="s">
+        <v>28</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>7</v>
+      </c>
+      <c r="B53" s="4">
+        <f t="shared" ref="B53:B54" si="14">ROW(A52)</f>
+        <v>52</v>
+      </c>
+      <c r="C53" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D53" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="E53" t="s">
+        <v>28</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>7</v>
+      </c>
+      <c r="B54" s="4">
+        <f t="shared" si="14"/>
+        <v>53</v>
+      </c>
+      <c r="C54" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D54" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="E54" t="s">
+        <v>28</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>7</v>
+      </c>
+      <c r="B55" s="4">
+        <f t="shared" ref="B55:B56" si="15">ROW(A54)</f>
+        <v>54</v>
+      </c>
+      <c r="C55" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D55" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="E55" t="s">
+        <v>28</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>7</v>
+      </c>
+      <c r="B56" s="4">
+        <f t="shared" si="15"/>
+        <v>55</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D56" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="E56" t="s">
+        <v>28</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>7</v>
+      </c>
+      <c r="B57" s="4">
+        <f t="shared" ref="B57:B58" si="16">ROW(A56)</f>
+        <v>56</v>
+      </c>
+      <c r="C57" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D57" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E57" t="s">
+        <v>28</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>7</v>
+      </c>
+      <c r="B58" s="4">
+        <f t="shared" si="16"/>
+        <v>57</v>
+      </c>
+      <c r="C58" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D58" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="E58" t="s">
+        <v>28</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>7</v>
+      </c>
+      <c r="B59" s="4">
+        <f t="shared" ref="B59:B60" si="17">ROW(A58)</f>
+        <v>58</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="E59" t="s">
+        <v>28</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>7</v>
+      </c>
+      <c r="B60" s="4">
+        <f t="shared" si="17"/>
+        <v>59</v>
+      </c>
+      <c r="C60" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="E60" t="s">
+        <v>28</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>7</v>
+      </c>
+      <c r="B61" s="4">
+        <f t="shared" ref="B61:B62" si="18">ROW(A60)</f>
+        <v>60</v>
+      </c>
+      <c r="C61" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D61" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="E61" t="s">
+        <v>28</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>7</v>
+      </c>
+      <c r="B62" s="4">
+        <f t="shared" si="18"/>
+        <v>61</v>
+      </c>
+      <c r="C62" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D62" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="E62" t="s">
+        <v>28</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>7</v>
+      </c>
+      <c r="B63" s="4">
+        <f t="shared" ref="B63:B64" si="19">ROW(A62)</f>
+        <v>62</v>
+      </c>
+      <c r="C63" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D63" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="E63" t="s">
+        <v>28</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>7</v>
+      </c>
+      <c r="B64" s="4">
+        <f t="shared" si="19"/>
+        <v>63</v>
+      </c>
+      <c r="C64" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D64" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="E64" t="s">
+        <v>28</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -1353,25 +2322,25 @@
           <x14:formula1>
             <xm:f>dpt_delta!$A$2:$A$24</xm:f>
           </x14:formula1>
-          <xm:sqref>A31:A52 F31:F52</xm:sqref>
+          <xm:sqref>A67:A88</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Código de la dpt de parroquia" prompt="Código de la dpt de parroquia">
           <x14:formula1>
             <xm:f>dpt_delta!$A$2:$A$24</xm:f>
           </x14:formula1>
-          <xm:sqref>A29:A30 A1 F1:F30</xm:sqref>
+          <xm:sqref>A65:A66 A1</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>dpt_delta!$B$2:$B$24</xm:f>
           </x14:formula1>
-          <xm:sqref>A2:A28</xm:sqref>
+          <xm:sqref>A2:A64</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Formato de la Publicación" prompt="Formato de la Publicación">
           <x14:formula1>
             <xm:f>formato!$A$2:$A$12</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E28</xm:sqref>
+          <xm:sqref>E2:E64</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1389,16 +2358,16 @@
         <v>25</v>
       </c>
       <c r="B1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" t="s">
         <v>30</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>31</v>
       </c>
-      <c r="D1" t="s">
-        <v>32</v>
-      </c>
       <c r="E1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -1618,62 +2587,62 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se agrego curiapo y el resto de padre baral
</commit_message>
<xml_diff>
--- a/libro_publicaciones.xlsx
+++ b/libro_publicaciones.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="753" uniqueCount="326">
   <si>
     <t>codigo</t>
   </si>
@@ -537,6 +537,474 @@
   </si>
   <si>
     <t>https://drive.google.com/file/d/1PzvKm47faiNB3g73QdKmLGO8Uqg6KMr9/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA ARIWINI</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1orkbBXh-fO9Z2f8NtUkmIgPAsOUNRENu/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1HLxYZuXswsU6SqpWmwU8QyUCfp0UfzWn/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA ISLA NUEVA</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA NOIMA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1Qh8Fr1qfZ2eMblPPkt67oQNFg70zq5j9/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA BOCA DE WUAKUJANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1R6_rXEoemtNqGs3WeVITYyuiywEzJklp/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA JOTUIDA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1Rmfslc7BentE-2R5t7JYkePmfbHnY-ZU/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA CAÑO NOIMA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1ylAF5UJGElSsqv7nBpT18vU0OS3_kxIK/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA WAKUJANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1xfHjcy_LH_-yat0-d0r21Kz0mHNVu543/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA JOJOBUNOKO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/10TJ5QXgr5LtdwXhravASCL5dVBJt9cOa/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA AUNO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1xsKrHEDbqmU_ncFEQDWY_5elvV61kshL/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA BELLA VISTA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1IKlVGOaI_b3gNcXHU_QqKRzw1oOULj1o/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA LA LECHOZA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1NXKFuYMULzpjFdjQ6Y9a-E30SpUl668B/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA DAWAJAKABANOKO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1cY_JT3jRivjrtMUbg6DK1fBPn_FhCJFm/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1tgcZbMyN5wPhyBD-nrqMOQKhYwwF5k_-/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA CURIAPITO II</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1eWvH7TJU4pVut15AsILBJUbP4oBoKL5D/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA PERICO</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA BAJOROBAKA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1BqhWyCpNs-r9zQuG4wlbTaHT2Kmp6bY2/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA TECOJANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1box69g2aWiMEYP9j1EIiZG2NKCgDPpot/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA ABAJA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/10fvUGT_l46bEootHQ_qf_00km8Trh3le/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA LOS REMOLINOS</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1iGCpIt8hfakXw9KGPMAemEI2nhKDR8uH/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA BOCA YAKURE</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1HC-v6JPKmFXk9focZSfv4_2N_4xTonYQ/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA IKAWARITO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/15m83i3Tg5jzqogT1Z3_g8nSewIHqjsdG/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA JOMATUBU</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1SL_IxJcNiwV8ENvdgNnaJoXFcn_XT_yn/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA JANEIDA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/11K1v-GEIRFNMoKGYQBokenkoX-lXefDS/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA LOS TRES CAÑOS</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/14Vht7vfIs7BRPlyEmuNPxbuijaUSfm9m/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA OTUIDA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1ga4UtqywWn0GZPcryGLPg5QTaBpv0M3e/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA MABORO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1zq0cgjkYDKoxnBMwh9HSxqOmGqJ5MQVM/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA WAJANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1zx2Q8u4LiXifN383sKiZBdGbgKZZKDS0/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA MUASIMOINA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/11drjKcJwrgnQ2fpy07BtL5p3rvkowwh_/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA LOS TIGRITOS</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1RBpmSffVfMQr0zY0o6hLHhsqyDcXfxl3/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA AIBE</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1YYHwagDyUcm0NFQUMV4Y2hDErhDTEg2W/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA LAS PIEDRITAS</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1e7gyF_T7J4yF0IU548x7dxoQB2_nAud8/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  JAJERUINA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/11r6EYM9_fyoZEVK4NN_ZKJrkBTkMQSC8/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  IKAWARE</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/17K_vKbB5AjjCL_ITzOfMSUgPaIl8MW5N/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  CANGREJITO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/14rIP308U4Al1G5x5U96hHTZtKCoAvr8l/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  WARAKASANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/18RMbmJMv1v3MQEe7LgZmMznR2T6AlJ93/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  KAJUNOKO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1LmQhR5ohTFug8IwV296yyOM2lMPj86C4/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA CURIAPITO I</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1gqHyoqKSX-yPpxj5PhRO2n2mTg4UCosr/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA PAGAYOS</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1PTf4qNvUJoRA8pun9dSmHaL8DX1TnwRr/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA YABAOVAKA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1qKmRl4-i0Ug1JPGIdrlv7SvPQo6mSSlo/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA SIMOKONOIMA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1EvngxjLa5Wfax4-n_fjotlDC00GZ6jA6/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA YEINAJANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1Z_BlwcCpN54DNw_gaet9J-MVY3mrNQP4/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA KAJAKARI</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1v505Eq0c4sQQgaKHV4csEmVqycqxeffH/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA IBARUMA I</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1CMnY4p_OM1s1aPjUUqczsaTvUu3tYOIE/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  JOYOJANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1d4vX0tv5v7iJDVdJxnjpHamQlZopUhSb/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  DOMUSIBU II</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/14rWeGDgSFQfYWEzz9lPU3oJwDeFmEKXq/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  RIO GRANDE</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1X_Pcsxc7ofLso_MJgUFd7mHdFH7y_e_C/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  SIMOA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1qQkSzyO97_iljFw__veyt5fbK1QP05Vd/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  JARUBUTONOKO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/10VpMZfgPAXdtI60SA9gXYJxKXLTs7dkm/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  JOKABANOKO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/10Y-a5I9lhBTXuCkySJHVj5b6ik5XVnGP/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  JUANAKASI</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1fWbGjD0qW8MVaIUF0wFcYdwYPIpbNOZw/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  WINAJANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1DToc5TkIa42iBsKL5xRSfHldawGZ2D33/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  MAYOR DOMO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1IQwnvbe_8BH2uLiuVu97PuW-p9YN9lKd/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  IBARUMA II</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1HZ5DwTDp_G06Ckx209JW1buGMfy0w25R/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  BOCA DE ARATURE</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1010Dsfgz_gT_9cSTvT_KZM6uIu0Xr2EB/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  PLAYA MUASIMOINA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1fD4CnDXBe5N_bNgL6uN2VAtaPrsmdDWA/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/10epcFjovirqB7X4jh4Y6ZtKzBlHtFpw_/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  LA KATAÑA </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  YORIKAJAMANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1JzOrpKWSXXS4w2hEV-zdss_w8qm_1JBq/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  WASIBOROJO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1IiSy7DEBT6FgPKV053j1k7XD6Wm16WLR/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  YOJANATINOKO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1GdqxD5ubjAFNSYT5yZzwN4YCV0_eBFTp/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  KOJUDOKOIDA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1SWX-mC1XNYtE7vaFLIhgXjjHK_RiYm7e/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  LAS MARGARITAS</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1FWUCuBpfs-8IbOCQOzOMOwdjHmh69soR/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1eBCFsGDRrLzFzsdlfcTx5ayGtCGCGLI9/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA   BABEJANA</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA SANTA TERESA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1WP77SMNQq-1MCaWL7cCnhAdHKzrRMvJL/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA DOMUSIBU I</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1YamAeeQYj079Sl3pdYSv7AVWnRm9e83c/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA KUAMUJO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/10ZLgxT3s-gkOwZq8fYgTQVrFibTxnV2X/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA AYARINA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/16u3X0mjgeMzCWSocdNglj4bNY5sr5Qdn/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA ITAJEREINA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1-OFczp3utuDs9iskf--AcTGlRttBtOji/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA SAN RAFAEL</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1aBdfleVDuh9P55y-EZHUnoF6cWyggYXs/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA BOCA COJINA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1U2sozOeVGA7eIbqU6hVV1o28JByiF7Fs/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA JOBURE II</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1dBBm9BzbTQF_YgwPlUmy2iHg5DHHo54b/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA LA MORA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1BSVGg3wFICp3ETws7Az7-JtHCiPpXBqi/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  JANAMANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1xpRgaj-9hWPGCxBO6xMDXrbPM2xg3s9q/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  JOBURE I</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1kT0wHnHtkUGvNRlKzWUi8MmSlrHoX1DV/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  DEJENEINA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/12J8J-pdxHbaY_8ljxznOj7cuoO6ByNdU/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  MEREJINA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1YqknjPq02U5KvsNqgmzvj8lnOJCPKPha/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  KAIWIRE</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1T-mRFPQnMIxpeXwtw7sj20HxwhoELgzn/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  MAJIKA DE MEREJINA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1jSn2XE1ceLy3wAtfXNrlZWvyMTtzP7EU/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  MUSEREINA DE COJINA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1QIxnvo9OP1gJUFG6F7QlZtFmOIMBea4N/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  KUAMUJO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1iuTz6PDcymXfCufEEgxJeK__jghSifVf/view?usp=drive_link</t>
   </si>
 </sst>
 </file>
@@ -676,8 +1144,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:F64" totalsRowShown="0">
-  <autoFilter ref="A1:F64"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:F142" totalsRowShown="0">
+  <autoFilter ref="A1:F142"/>
   <tableColumns count="6">
     <tableColumn id="1" name="cod_dpt"/>
     <tableColumn id="2" name="cod_publicacion" dataDxfId="2">
@@ -955,7 +1423,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F142"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -2309,6 +2777,1644 @@
         <v>169</v>
       </c>
     </row>
+    <row r="65" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>3</v>
+      </c>
+      <c r="B65" s="4">
+        <f t="shared" ref="B65:B66" si="20">ROW(A64)</f>
+        <v>64</v>
+      </c>
+      <c r="C65" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D65" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="E65" t="s">
+        <v>28</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>3</v>
+      </c>
+      <c r="B66" s="4">
+        <f t="shared" si="20"/>
+        <v>65</v>
+      </c>
+      <c r="C66" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D66" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="E66" t="s">
+        <v>28</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>3</v>
+      </c>
+      <c r="B67" s="4">
+        <f t="shared" ref="B67:B68" si="21">ROW(A66)</f>
+        <v>66</v>
+      </c>
+      <c r="C67" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D67" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E67" t="s">
+        <v>28</v>
+      </c>
+      <c r="F67" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>3</v>
+      </c>
+      <c r="B68" s="4">
+        <f t="shared" si="21"/>
+        <v>67</v>
+      </c>
+      <c r="C68" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D68" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="E68" t="s">
+        <v>28</v>
+      </c>
+      <c r="F68" s="1" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>3</v>
+      </c>
+      <c r="B69" s="4">
+        <f t="shared" ref="B69:B70" si="22">ROW(A68)</f>
+        <v>68</v>
+      </c>
+      <c r="C69" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D69" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="E69" t="s">
+        <v>28</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>3</v>
+      </c>
+      <c r="B70" s="4">
+        <f t="shared" si="22"/>
+        <v>69</v>
+      </c>
+      <c r="C70" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D70" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="E70" t="s">
+        <v>28</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>3</v>
+      </c>
+      <c r="B71" s="4">
+        <f t="shared" ref="B71:B72" si="23">ROW(A70)</f>
+        <v>70</v>
+      </c>
+      <c r="C71" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D71" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="E71" t="s">
+        <v>28</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>3</v>
+      </c>
+      <c r="B72" s="4">
+        <f t="shared" si="23"/>
+        <v>71</v>
+      </c>
+      <c r="C72" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D72" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="E72" t="s">
+        <v>28</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>3</v>
+      </c>
+      <c r="B73" s="4">
+        <f t="shared" ref="B73" si="24">ROW(A72)</f>
+        <v>72</v>
+      </c>
+      <c r="C73" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D73" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="E73" t="s">
+        <v>28</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>3</v>
+      </c>
+      <c r="B74" s="4">
+        <f t="shared" ref="B74" si="25">ROW(A73)</f>
+        <v>73</v>
+      </c>
+      <c r="C74" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D74" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="E74" t="s">
+        <v>28</v>
+      </c>
+      <c r="F74" s="1" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>3</v>
+      </c>
+      <c r="B75" s="4">
+        <f t="shared" ref="B75" si="26">ROW(A74)</f>
+        <v>74</v>
+      </c>
+      <c r="C75" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D75" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="E75" t="s">
+        <v>28</v>
+      </c>
+      <c r="F75" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>3</v>
+      </c>
+      <c r="B76" s="4">
+        <f t="shared" ref="B76" si="27">ROW(A75)</f>
+        <v>75</v>
+      </c>
+      <c r="C76" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D76" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="E76" t="s">
+        <v>28</v>
+      </c>
+      <c r="F76" s="1" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>3</v>
+      </c>
+      <c r="B77" s="4">
+        <f t="shared" ref="B77" si="28">ROW(A76)</f>
+        <v>76</v>
+      </c>
+      <c r="C77" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D77" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="E77" t="s">
+        <v>28</v>
+      </c>
+      <c r="F77" s="1" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>3</v>
+      </c>
+      <c r="B78" s="4">
+        <f t="shared" ref="B78" si="29">ROW(A77)</f>
+        <v>77</v>
+      </c>
+      <c r="C78" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D78" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="E78" t="s">
+        <v>28</v>
+      </c>
+      <c r="F78" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>3</v>
+      </c>
+      <c r="B79" s="4">
+        <f t="shared" ref="B79" si="30">ROW(A78)</f>
+        <v>78</v>
+      </c>
+      <c r="C79" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D79" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="E79" t="s">
+        <v>28</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>3</v>
+      </c>
+      <c r="B80" s="4">
+        <f t="shared" ref="B80" si="31">ROW(A79)</f>
+        <v>79</v>
+      </c>
+      <c r="C80" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D80" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="E80" t="s">
+        <v>28</v>
+      </c>
+      <c r="F80" s="1" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>3</v>
+      </c>
+      <c r="B81" s="4">
+        <f t="shared" ref="B81" si="32">ROW(A80)</f>
+        <v>80</v>
+      </c>
+      <c r="C81" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D81" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="E81" t="s">
+        <v>28</v>
+      </c>
+      <c r="F81" s="1" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>3</v>
+      </c>
+      <c r="B82" s="4">
+        <f t="shared" ref="B82" si="33">ROW(A81)</f>
+        <v>81</v>
+      </c>
+      <c r="C82" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D82" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="E82" t="s">
+        <v>28</v>
+      </c>
+      <c r="F82" s="1" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>3</v>
+      </c>
+      <c r="B83" s="4">
+        <f t="shared" ref="B83" si="34">ROW(A82)</f>
+        <v>82</v>
+      </c>
+      <c r="C83" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D83" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="E83" t="s">
+        <v>28</v>
+      </c>
+      <c r="F83" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>3</v>
+      </c>
+      <c r="B84" s="4">
+        <f t="shared" ref="B84" si="35">ROW(A83)</f>
+        <v>83</v>
+      </c>
+      <c r="C84" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D84" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="E84" t="s">
+        <v>28</v>
+      </c>
+      <c r="F84" s="1" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>3</v>
+      </c>
+      <c r="B85" s="4">
+        <f t="shared" ref="B85" si="36">ROW(A84)</f>
+        <v>84</v>
+      </c>
+      <c r="C85" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D85" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="E85" t="s">
+        <v>28</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>3</v>
+      </c>
+      <c r="B86" s="4">
+        <f t="shared" ref="B86" si="37">ROW(A85)</f>
+        <v>85</v>
+      </c>
+      <c r="C86" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D86" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="E86" t="s">
+        <v>28</v>
+      </c>
+      <c r="F86" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>3</v>
+      </c>
+      <c r="B87" s="4">
+        <f t="shared" ref="B87" si="38">ROW(A86)</f>
+        <v>86</v>
+      </c>
+      <c r="C87" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D87" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="E87" t="s">
+        <v>28</v>
+      </c>
+      <c r="F87" s="1" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>3</v>
+      </c>
+      <c r="B88" s="4">
+        <f t="shared" ref="B88" si="39">ROW(A87)</f>
+        <v>87</v>
+      </c>
+      <c r="C88" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D88" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="E88" t="s">
+        <v>28</v>
+      </c>
+      <c r="F88" s="1" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>3</v>
+      </c>
+      <c r="B89" s="4">
+        <f t="shared" ref="B89" si="40">ROW(A88)</f>
+        <v>88</v>
+      </c>
+      <c r="C89" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D89" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="E89" t="s">
+        <v>28</v>
+      </c>
+      <c r="F89" s="1" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>3</v>
+      </c>
+      <c r="B90" s="4">
+        <f t="shared" ref="B90" si="41">ROW(A89)</f>
+        <v>89</v>
+      </c>
+      <c r="C90" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D90" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="E90" t="s">
+        <v>28</v>
+      </c>
+      <c r="F90" s="1" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>3</v>
+      </c>
+      <c r="B91" s="4">
+        <f t="shared" ref="B91" si="42">ROW(A90)</f>
+        <v>90</v>
+      </c>
+      <c r="C91" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D91" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="E91" t="s">
+        <v>28</v>
+      </c>
+      <c r="F91" s="1" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>3</v>
+      </c>
+      <c r="B92" s="4">
+        <f t="shared" ref="B92" si="43">ROW(A91)</f>
+        <v>91</v>
+      </c>
+      <c r="C92" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D92" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="E92" t="s">
+        <v>28</v>
+      </c>
+      <c r="F92" s="1" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>3</v>
+      </c>
+      <c r="B93" s="4">
+        <f t="shared" ref="B93" si="44">ROW(A92)</f>
+        <v>92</v>
+      </c>
+      <c r="C93" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D93" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="E93" t="s">
+        <v>28</v>
+      </c>
+      <c r="F93" s="1" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>3</v>
+      </c>
+      <c r="B94" s="4">
+        <f t="shared" ref="B94" si="45">ROW(A93)</f>
+        <v>93</v>
+      </c>
+      <c r="C94" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D94" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="E94" t="s">
+        <v>28</v>
+      </c>
+      <c r="F94" s="1" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>3</v>
+      </c>
+      <c r="B95" s="4">
+        <f t="shared" ref="B95" si="46">ROW(A94)</f>
+        <v>94</v>
+      </c>
+      <c r="C95" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D95" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="E95" t="s">
+        <v>28</v>
+      </c>
+      <c r="F95" s="1" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>3</v>
+      </c>
+      <c r="B96" s="4">
+        <f t="shared" ref="B96" si="47">ROW(A95)</f>
+        <v>95</v>
+      </c>
+      <c r="C96" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D96" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="E96" t="s">
+        <v>28</v>
+      </c>
+      <c r="F96" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>3</v>
+      </c>
+      <c r="B97" s="4">
+        <f t="shared" ref="B97" si="48">ROW(A96)</f>
+        <v>96</v>
+      </c>
+      <c r="C97" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D97" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="E97" t="s">
+        <v>28</v>
+      </c>
+      <c r="F97" s="1" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>3</v>
+      </c>
+      <c r="B98" s="4">
+        <f t="shared" ref="B98" si="49">ROW(A97)</f>
+        <v>97</v>
+      </c>
+      <c r="C98" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D98" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="E98" t="s">
+        <v>28</v>
+      </c>
+      <c r="F98" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>3</v>
+      </c>
+      <c r="B99" s="4">
+        <f t="shared" ref="B99" si="50">ROW(A98)</f>
+        <v>98</v>
+      </c>
+      <c r="C99" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D99" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="E99" t="s">
+        <v>28</v>
+      </c>
+      <c r="F99" s="1" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>3</v>
+      </c>
+      <c r="B100" s="4">
+        <f t="shared" ref="B100" si="51">ROW(A99)</f>
+        <v>99</v>
+      </c>
+      <c r="C100" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D100" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="E100" t="s">
+        <v>28</v>
+      </c>
+      <c r="F100" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>3</v>
+      </c>
+      <c r="B101" s="4">
+        <f t="shared" ref="B101" si="52">ROW(A100)</f>
+        <v>100</v>
+      </c>
+      <c r="C101" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D101" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="E101" t="s">
+        <v>28</v>
+      </c>
+      <c r="F101" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>3</v>
+      </c>
+      <c r="B102" s="4">
+        <f t="shared" ref="B102" si="53">ROW(A101)</f>
+        <v>101</v>
+      </c>
+      <c r="C102" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D102" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="E102" t="s">
+        <v>28</v>
+      </c>
+      <c r="F102" s="1" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>3</v>
+      </c>
+      <c r="B103" s="4">
+        <f t="shared" ref="B103" si="54">ROW(A102)</f>
+        <v>102</v>
+      </c>
+      <c r="C103" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D103" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="E103" t="s">
+        <v>28</v>
+      </c>
+      <c r="F103" s="1" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>3</v>
+      </c>
+      <c r="B104" s="4">
+        <f t="shared" ref="B104" si="55">ROW(A103)</f>
+        <v>103</v>
+      </c>
+      <c r="C104" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D104" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="E104" t="s">
+        <v>28</v>
+      </c>
+      <c r="F104" s="1" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>3</v>
+      </c>
+      <c r="B105" s="4">
+        <f t="shared" ref="B105" si="56">ROW(A104)</f>
+        <v>104</v>
+      </c>
+      <c r="C105" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D105" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="E105" t="s">
+        <v>28</v>
+      </c>
+      <c r="F105" s="1" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>3</v>
+      </c>
+      <c r="B106" s="4">
+        <f t="shared" ref="B106" si="57">ROW(A105)</f>
+        <v>105</v>
+      </c>
+      <c r="C106" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D106" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="E106" t="s">
+        <v>28</v>
+      </c>
+      <c r="F106" s="1" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>3</v>
+      </c>
+      <c r="B107" s="4">
+        <f t="shared" ref="B107" si="58">ROW(A106)</f>
+        <v>106</v>
+      </c>
+      <c r="C107" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D107" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="E107" t="s">
+        <v>28</v>
+      </c>
+      <c r="F107" s="1" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>3</v>
+      </c>
+      <c r="B108" s="4">
+        <f t="shared" ref="B108" si="59">ROW(A107)</f>
+        <v>107</v>
+      </c>
+      <c r="C108" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D108" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="E108" t="s">
+        <v>28</v>
+      </c>
+      <c r="F108" s="1" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>3</v>
+      </c>
+      <c r="B109" s="4">
+        <f t="shared" ref="B109" si="60">ROW(A108)</f>
+        <v>108</v>
+      </c>
+      <c r="C109" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D109" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="E109" t="s">
+        <v>28</v>
+      </c>
+      <c r="F109" s="1" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>3</v>
+      </c>
+      <c r="B110" s="4">
+        <f t="shared" ref="B110" si="61">ROW(A109)</f>
+        <v>109</v>
+      </c>
+      <c r="C110" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D110" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="E110" t="s">
+        <v>28</v>
+      </c>
+      <c r="F110" s="1" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>3</v>
+      </c>
+      <c r="B111" s="4">
+        <f t="shared" ref="B111" si="62">ROW(A110)</f>
+        <v>110</v>
+      </c>
+      <c r="C111" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D111" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="E111" t="s">
+        <v>28</v>
+      </c>
+      <c r="F111" s="1" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>3</v>
+      </c>
+      <c r="B112" s="4">
+        <f t="shared" ref="B112" si="63">ROW(A111)</f>
+        <v>111</v>
+      </c>
+      <c r="C112" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D112" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="E112" t="s">
+        <v>28</v>
+      </c>
+      <c r="F112" s="1" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>3</v>
+      </c>
+      <c r="B113" s="4">
+        <f t="shared" ref="B113" si="64">ROW(A112)</f>
+        <v>112</v>
+      </c>
+      <c r="C113" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D113" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="E113" t="s">
+        <v>28</v>
+      </c>
+      <c r="F113" s="1" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>3</v>
+      </c>
+      <c r="B114" s="4">
+        <f t="shared" ref="B114" si="65">ROW(A113)</f>
+        <v>113</v>
+      </c>
+      <c r="C114" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D114" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="E114" t="s">
+        <v>28</v>
+      </c>
+      <c r="F114" s="1" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>3</v>
+      </c>
+      <c r="B115" s="4">
+        <f t="shared" ref="B115" si="66">ROW(A114)</f>
+        <v>114</v>
+      </c>
+      <c r="C115" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D115" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="E115" t="s">
+        <v>28</v>
+      </c>
+      <c r="F115" s="1" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>3</v>
+      </c>
+      <c r="B116" s="4">
+        <f t="shared" ref="B116" si="67">ROW(A115)</f>
+        <v>115</v>
+      </c>
+      <c r="C116" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D116" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="E116" t="s">
+        <v>28</v>
+      </c>
+      <c r="F116" s="1" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>3</v>
+      </c>
+      <c r="B117" s="4">
+        <f t="shared" ref="B117" si="68">ROW(A116)</f>
+        <v>116</v>
+      </c>
+      <c r="C117" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D117" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="E117" t="s">
+        <v>28</v>
+      </c>
+      <c r="F117" s="1" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>3</v>
+      </c>
+      <c r="B118" s="4">
+        <f t="shared" ref="B118" si="69">ROW(A117)</f>
+        <v>117</v>
+      </c>
+      <c r="C118" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D118" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="E118" t="s">
+        <v>28</v>
+      </c>
+      <c r="F118" s="1" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>3</v>
+      </c>
+      <c r="B119" s="4">
+        <f t="shared" ref="B119" si="70">ROW(A118)</f>
+        <v>118</v>
+      </c>
+      <c r="C119" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D119" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="E119" t="s">
+        <v>28</v>
+      </c>
+      <c r="F119" s="1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>3</v>
+      </c>
+      <c r="B120" s="4">
+        <f t="shared" ref="B120" si="71">ROW(A119)</f>
+        <v>119</v>
+      </c>
+      <c r="C120" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D120" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="E120" t="s">
+        <v>28</v>
+      </c>
+      <c r="F120" s="1" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>3</v>
+      </c>
+      <c r="B121" s="4">
+        <f t="shared" ref="B121" si="72">ROW(A120)</f>
+        <v>120</v>
+      </c>
+      <c r="C121" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D121" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="E121" t="s">
+        <v>28</v>
+      </c>
+      <c r="F121" s="1" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>3</v>
+      </c>
+      <c r="B122" s="4">
+        <f t="shared" ref="B122" si="73">ROW(A121)</f>
+        <v>121</v>
+      </c>
+      <c r="C122" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D122" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="E122" t="s">
+        <v>28</v>
+      </c>
+      <c r="F122" s="1" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>3</v>
+      </c>
+      <c r="B123" s="4">
+        <f t="shared" ref="B123" si="74">ROW(A122)</f>
+        <v>122</v>
+      </c>
+      <c r="C123" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D123" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="E123" t="s">
+        <v>28</v>
+      </c>
+      <c r="F123" s="1" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>3</v>
+      </c>
+      <c r="B124" s="4">
+        <f t="shared" ref="B124" si="75">ROW(A123)</f>
+        <v>123</v>
+      </c>
+      <c r="C124" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D124" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="E124" t="s">
+        <v>28</v>
+      </c>
+      <c r="F124" s="1" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>3</v>
+      </c>
+      <c r="B125" s="4">
+        <f t="shared" ref="B125" si="76">ROW(A124)</f>
+        <v>124</v>
+      </c>
+      <c r="C125" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D125" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="E125" t="s">
+        <v>28</v>
+      </c>
+      <c r="F125" s="1" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>3</v>
+      </c>
+      <c r="B126" s="4">
+        <f t="shared" ref="B126" si="77">ROW(A125)</f>
+        <v>125</v>
+      </c>
+      <c r="C126" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D126" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="E126" t="s">
+        <v>28</v>
+      </c>
+      <c r="F126" s="1" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>3</v>
+      </c>
+      <c r="B127" s="4">
+        <f t="shared" ref="B127" si="78">ROW(A126)</f>
+        <v>126</v>
+      </c>
+      <c r="C127" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D127" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="E127" t="s">
+        <v>28</v>
+      </c>
+      <c r="F127" s="1" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>3</v>
+      </c>
+      <c r="B128" s="4">
+        <f t="shared" ref="B128" si="79">ROW(A127)</f>
+        <v>127</v>
+      </c>
+      <c r="C128" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D128" s="5" t="s">
+        <v>296</v>
+      </c>
+      <c r="E128" t="s">
+        <v>28</v>
+      </c>
+      <c r="F128" s="1" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>3</v>
+      </c>
+      <c r="B129" s="4">
+        <f t="shared" ref="B129" si="80">ROW(A128)</f>
+        <v>128</v>
+      </c>
+      <c r="C129" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D129" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="E129" t="s">
+        <v>28</v>
+      </c>
+      <c r="F129" s="1" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>3</v>
+      </c>
+      <c r="B130" s="4">
+        <f t="shared" ref="B130" si="81">ROW(A129)</f>
+        <v>129</v>
+      </c>
+      <c r="C130" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D130" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="E130" t="s">
+        <v>28</v>
+      </c>
+      <c r="F130" s="1" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>3</v>
+      </c>
+      <c r="B131" s="4">
+        <f t="shared" ref="B131" si="82">ROW(A130)</f>
+        <v>130</v>
+      </c>
+      <c r="C131" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D131" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="E131" t="s">
+        <v>28</v>
+      </c>
+      <c r="F131" s="1" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>7</v>
+      </c>
+      <c r="B132" s="4">
+        <f t="shared" ref="B132" si="83">ROW(A131)</f>
+        <v>131</v>
+      </c>
+      <c r="C132" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D132" s="5" t="s">
+        <v>304</v>
+      </c>
+      <c r="E132" t="s">
+        <v>28</v>
+      </c>
+      <c r="F132" s="1" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>7</v>
+      </c>
+      <c r="B133" s="4">
+        <f t="shared" ref="B133" si="84">ROW(A132)</f>
+        <v>132</v>
+      </c>
+      <c r="C133" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D133" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="E133" t="s">
+        <v>28</v>
+      </c>
+      <c r="F133" s="1" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>7</v>
+      </c>
+      <c r="B134" s="4">
+        <f t="shared" ref="B134" si="85">ROW(A133)</f>
+        <v>133</v>
+      </c>
+      <c r="C134" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D134" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="E134" t="s">
+        <v>28</v>
+      </c>
+      <c r="F134" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>7</v>
+      </c>
+      <c r="B135" s="4">
+        <f t="shared" ref="B135" si="86">ROW(A134)</f>
+        <v>134</v>
+      </c>
+      <c r="C135" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D135" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="E135" t="s">
+        <v>28</v>
+      </c>
+      <c r="F135" s="1" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>7</v>
+      </c>
+      <c r="B136" s="4">
+        <f t="shared" ref="B136" si="87">ROW(A135)</f>
+        <v>135</v>
+      </c>
+      <c r="C136" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D136" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="E136" t="s">
+        <v>28</v>
+      </c>
+      <c r="F136" s="1" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>7</v>
+      </c>
+      <c r="B137" s="4">
+        <f t="shared" ref="B137" si="88">ROW(A136)</f>
+        <v>136</v>
+      </c>
+      <c r="C137" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D137" s="5" t="s">
+        <v>314</v>
+      </c>
+      <c r="E137" t="s">
+        <v>28</v>
+      </c>
+      <c r="F137" s="1" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>7</v>
+      </c>
+      <c r="B138" s="4">
+        <f t="shared" ref="B138" si="89">ROW(A137)</f>
+        <v>137</v>
+      </c>
+      <c r="C138" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D138" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="E138" t="s">
+        <v>28</v>
+      </c>
+      <c r="F138" s="1" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>7</v>
+      </c>
+      <c r="B139" s="4">
+        <f t="shared" ref="B139" si="90">ROW(A138)</f>
+        <v>138</v>
+      </c>
+      <c r="C139" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D139" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="E139" t="s">
+        <v>28</v>
+      </c>
+      <c r="F139" s="1" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>7</v>
+      </c>
+      <c r="B140" s="4">
+        <f t="shared" ref="B140" si="91">ROW(A139)</f>
+        <v>139</v>
+      </c>
+      <c r="C140" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D140" s="5" t="s">
+        <v>320</v>
+      </c>
+      <c r="E140" t="s">
+        <v>28</v>
+      </c>
+      <c r="F140" s="1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>7</v>
+      </c>
+      <c r="B141" s="4">
+        <f t="shared" ref="B141" si="92">ROW(A140)</f>
+        <v>140</v>
+      </c>
+      <c r="C141" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D141" s="5" t="s">
+        <v>322</v>
+      </c>
+      <c r="E141" t="s">
+        <v>28</v>
+      </c>
+      <c r="F141" s="1" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>7</v>
+      </c>
+      <c r="B142" s="4">
+        <f t="shared" ref="B142" si="93">ROW(A141)</f>
+        <v>141</v>
+      </c>
+      <c r="C142" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D142" s="5" t="s">
+        <v>324</v>
+      </c>
+      <c r="E142" t="s">
+        <v>28</v>
+      </c>
+      <c r="F142" s="1" t="s">
+        <v>325</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2322,25 +4428,25 @@
           <x14:formula1>
             <xm:f>dpt_delta!$A$2:$A$24</xm:f>
           </x14:formula1>
-          <xm:sqref>A67:A88</xm:sqref>
+          <xm:sqref>A145:A166</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Código de la dpt de parroquia" prompt="Código de la dpt de parroquia">
           <x14:formula1>
             <xm:f>dpt_delta!$A$2:$A$24</xm:f>
           </x14:formula1>
-          <xm:sqref>A65:A66 A1</xm:sqref>
+          <xm:sqref>A143:A144 A1</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>dpt_delta!$B$2:$B$24</xm:f>
           </x14:formula1>
-          <xm:sqref>A2:A64</xm:sqref>
+          <xm:sqref>A2:A142</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Formato de la Publicación" prompt="Formato de la Publicación">
           <x14:formula1>
             <xm:f>formato!$A$2:$A$12</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E64</xm:sqref>
+          <xm:sqref>E2:E142</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Se agrego una actualización de la parroquia santos albergas
</commit_message>
<xml_diff>
--- a/libro_publicaciones.xlsx
+++ b/libro_publicaciones.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fguedez\Documents\Proyectos\page-estadisticas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fguedez\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7905"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21600" windowHeight="9885"/>
   </bookViews>
   <sheets>
     <sheet name="data_parroquia" sheetId="2" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="753" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="798" uniqueCount="344">
   <si>
     <t>codigo</t>
   </si>
@@ -323,48 +323,6 @@
     <t>https://docs.google.com/presentation/d/1v354uD4Wq5tUS3q32K-7Tot1dqModJbb/edit?usp=drive_link&amp;ouid=105142876406402750370&amp;rtpof=true&amp;sd=true</t>
   </si>
   <si>
-    <t>https://drive.google.com/file/d/1kiGrAKpKFzvMIas5XiA-nwVBZ6ZCEX25/view?usp=drive_link</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/179KUodqofy8urV712zsOityyUree352T/view?usp=drive_link</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA Y CENTRO POBLADO BOCA DE ARAGUAO</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA Y CENTRO POBLADO POTRERITO</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA Y CENTRO POBLADO RAMANCE DE SACUPANA</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1IynOfRXoLoEg__G6RrzANlSGVftxjXaK/view?usp=drive_link</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA Y CENTRO JANAMANA</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1ojy5jD-Wlgcj1OvN_S8soiIRtKX15n9Y/view?usp=drive_link</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA Y CENTRO POBLADO BOCA DE SACUPANA</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1qGHkjsLvHRDloSnfztUOkQaoO2s61akh/view?usp=drive_link</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA Y CENTRO POBLADO CUBERINA</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1BopfCadXeFKi4oQrPdBS-G4PUZebq55q/view?usp=drive_link</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA Y CENTRO POBLADO ISLA EL NORTE</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1Ae_hTO6TSZNgDwwjQNxNcNC7vD5Ca-ZU/view?usp=drive_link</t>
-  </si>
-  <si>
     <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA DAUWARUBAKA</t>
   </si>
   <si>
@@ -1005,6 +963,102 @@
   </si>
   <si>
     <t>https://drive.google.com/file/d/1iuTz6PDcymXfCufEEgxJeK__jghSifVf/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA CRUCERO DE ARAGUAO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1MioZwDn-gIWaRKD9Lqi-LNMKi70bNAla/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA SANTA ROSA DE ARAGUAO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1ps8q89S-cKx8d149McJv-tNekWbcDPWI/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA ISLA EL NORTE</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1G-AGQ2MBkQLas8ObwsV3HtHSmM_2_q3d/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA SAN ANTONIO DE ARAGUAO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1ojRJBr-Xb4n6Rko8YKrA49Tt97ytE25J/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA POTRERITO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1ZfeMqez9BaXulsxMM9oPv418yOe-RxME/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA BOCA DEL CHORRO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1gjw7_6oRWPr3Wqgedushtj12Lolw83P0/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA LOS COCOS</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1i_qnaaCH9iY6dmZdS6uphWSSCz0_YwDT/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA BOCA DE SACUPANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1BywAVG8Auz3kXgYkrayvs3oOpfh9XvK5/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA REMANCE DE SACUPANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1bJjuj70espWnPt3VB55_JerwMh1FBC3Q/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA BOCA DE ARAGUAO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/13myBEg-kqPcCeqQBw-MedZi1fdQhdq3J/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA JANAMANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1FP3BgRR6Yivv5Tj1QwkCXzxllhuliS8c/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA ARAGUAIMUJO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1cVh0m6GJAv5W8rFN1D1N0vJjs52CQUDl/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA PUERTO LUIS</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1Hz5PalRt4Bpa1E2aAA3XHp3p6F6eG78P/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA JANAKASI</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1iF2-DZhH3jGKtNya81Ulf5ViS3jHHLnR/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA LOS MANGOS</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1wfOF7gwtaN6zCKb7vzLIT1i9NctXvHq-/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA CUBERINA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1Qe2iUdgGKJjrVDY1_0Cx7b4Gec0H0N1R/view?usp=drive_link</t>
   </si>
 </sst>
 </file>
@@ -1059,12 +1113,49 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -1073,7 +1164,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1084,6 +1175,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Énfasis1" xfId="2" builtinId="29"/>
@@ -1144,8 +1242,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:F142" totalsRowShown="0">
-  <autoFilter ref="A1:F142"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:F135" totalsRowShown="0">
+  <autoFilter ref="A1:F135"/>
   <tableColumns count="6">
     <tableColumn id="1" name="cod_dpt"/>
     <tableColumn id="2" name="cod_publicacion" dataDxfId="2">
@@ -1423,7 +1521,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F142"/>
+  <dimension ref="A1:J151"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1960,7 +2058,7 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="B26" s="4">
         <f t="shared" si="1"/>
@@ -2021,54 +2119,53 @@
         <v>97</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B29" s="4">
-        <f t="shared" ref="B29:B30" si="2">ROW(A28)</f>
         <v>28</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>55</v>
       </c>
       <c r="D29" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="E29" t="s">
+        <v>28</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>7</v>
+      </c>
+      <c r="B30" s="4">
+        <f t="shared" ref="B30:B31" si="2">ROW(A29)</f>
+        <v>29</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D30" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="E29" t="s">
-        <v>28</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>8</v>
-      </c>
-      <c r="B30" s="4">
+      <c r="E30" t="s">
+        <v>28</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>7</v>
+      </c>
+      <c r="B31" s="4">
         <f t="shared" si="2"/>
-        <v>29</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="E30" t="s">
-        <v>28</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>8</v>
-      </c>
-      <c r="B31" s="4">
-        <f t="shared" ref="B31:B32" si="3">ROW(A30)</f>
         <v>30</v>
       </c>
       <c r="C31" s="5" t="s">
@@ -2084,12 +2181,12 @@
         <v>103</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B32" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="B32:B33" si="3">ROW(A31)</f>
         <v>31</v>
       </c>
       <c r="C32" s="5" t="s">
@@ -2105,12 +2202,12 @@
         <v>105</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B33" s="4">
-        <f t="shared" ref="B33:B34" si="4">ROW(A32)</f>
+        <f t="shared" si="3"/>
         <v>32</v>
       </c>
       <c r="C33" s="5" t="s">
@@ -2126,12 +2223,12 @@
         <v>107</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B34" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="B34:B35" si="4">ROW(A33)</f>
         <v>33</v>
       </c>
       <c r="C34" s="5" t="s">
@@ -2147,12 +2244,12 @@
         <v>109</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B35" s="4">
-        <f t="shared" ref="B35:B36" si="5">ROW(A34)</f>
+        <f t="shared" si="4"/>
         <v>34</v>
       </c>
       <c r="C35" s="5" t="s">
@@ -2168,12 +2265,12 @@
         <v>111</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>7</v>
       </c>
       <c r="B36" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="B36:B37" si="5">ROW(A35)</f>
         <v>35</v>
       </c>
       <c r="C36" s="5" t="s">
@@ -2189,12 +2286,12 @@
         <v>113</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>7</v>
       </c>
       <c r="B37" s="4">
-        <f t="shared" ref="B37:B38" si="6">ROW(A36)</f>
+        <f t="shared" si="5"/>
         <v>36</v>
       </c>
       <c r="C37" s="5" t="s">
@@ -2210,12 +2307,12 @@
         <v>115</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>7</v>
       </c>
       <c r="B38" s="4">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="B38:B39" si="6">ROW(A37)</f>
         <v>37</v>
       </c>
       <c r="C38" s="5" t="s">
@@ -2231,12 +2328,12 @@
         <v>117</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>7</v>
       </c>
       <c r="B39" s="4">
-        <f t="shared" ref="B39:B40" si="7">ROW(A38)</f>
+        <f t="shared" si="6"/>
         <v>38</v>
       </c>
       <c r="C39" s="5" t="s">
@@ -2252,12 +2349,12 @@
         <v>119</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>7</v>
       </c>
       <c r="B40" s="4">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="B40:B41" si="7">ROW(A39)</f>
         <v>39</v>
       </c>
       <c r="C40" s="5" t="s">
@@ -2273,12 +2370,12 @@
         <v>121</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>7</v>
       </c>
       <c r="B41" s="4">
-        <f t="shared" ref="B41:B42" si="8">ROW(A40)</f>
+        <f t="shared" si="7"/>
         <v>40</v>
       </c>
       <c r="C41" s="5" t="s">
@@ -2294,12 +2391,12 @@
         <v>123</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>7</v>
       </c>
       <c r="B42" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="B42:B43" si="8">ROW(A41)</f>
         <v>41</v>
       </c>
       <c r="C42" s="5" t="s">
@@ -2315,12 +2412,12 @@
         <v>125</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>7</v>
       </c>
       <c r="B43" s="4">
-        <f t="shared" ref="B43:B44" si="9">ROW(A42)</f>
+        <f t="shared" si="8"/>
         <v>42</v>
       </c>
       <c r="C43" s="5" t="s">
@@ -2336,12 +2433,12 @@
         <v>127</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>7</v>
       </c>
       <c r="B44" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="B44:B45" si="9">ROW(A43)</f>
         <v>43</v>
       </c>
       <c r="C44" s="5" t="s">
@@ -2357,12 +2454,12 @@
         <v>129</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>7</v>
       </c>
       <c r="B45" s="4">
-        <f t="shared" ref="B45:B46" si="10">ROW(A44)</f>
+        <f t="shared" si="9"/>
         <v>44</v>
       </c>
       <c r="C45" s="5" t="s">
@@ -2378,12 +2475,12 @@
         <v>131</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>7</v>
       </c>
       <c r="B46" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" ref="B46:B47" si="10">ROW(A45)</f>
         <v>45</v>
       </c>
       <c r="C46" s="5" t="s">
@@ -2399,12 +2496,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>7</v>
       </c>
       <c r="B47" s="4">
-        <f t="shared" ref="B47:B48" si="11">ROW(A46)</f>
+        <f t="shared" si="10"/>
         <v>46</v>
       </c>
       <c r="C47" s="5" t="s">
@@ -2420,12 +2517,12 @@
         <v>135</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>7</v>
       </c>
       <c r="B48" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="B48:B49" si="11">ROW(A47)</f>
         <v>47</v>
       </c>
       <c r="C48" s="5" t="s">
@@ -2441,12 +2538,12 @@
         <v>137</v>
       </c>
     </row>
-    <row r="49" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>7</v>
       </c>
       <c r="B49" s="4">
-        <f t="shared" ref="B49:B50" si="12">ROW(A48)</f>
+        <f t="shared" si="11"/>
         <v>48</v>
       </c>
       <c r="C49" s="5" t="s">
@@ -2462,12 +2559,12 @@
         <v>139</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>7</v>
       </c>
       <c r="B50" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" ref="B50:B51" si="12">ROW(A49)</f>
         <v>49</v>
       </c>
       <c r="C50" s="5" t="s">
@@ -2483,12 +2580,12 @@
         <v>141</v>
       </c>
     </row>
-    <row r="51" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>7</v>
       </c>
       <c r="B51" s="4">
-        <f t="shared" ref="B51:B52" si="13">ROW(A50)</f>
+        <f t="shared" si="12"/>
         <v>50</v>
       </c>
       <c r="C51" s="5" t="s">
@@ -2504,12 +2601,12 @@
         <v>143</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>7</v>
       </c>
       <c r="B52" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" ref="B52:B53" si="13">ROW(A51)</f>
         <v>51</v>
       </c>
       <c r="C52" s="5" t="s">
@@ -2525,12 +2622,12 @@
         <v>145</v>
       </c>
     </row>
-    <row r="53" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>7</v>
       </c>
       <c r="B53" s="4">
-        <f t="shared" ref="B53:B54" si="14">ROW(A52)</f>
+        <f t="shared" si="13"/>
         <v>52</v>
       </c>
       <c r="C53" s="5" t="s">
@@ -2546,12 +2643,12 @@
         <v>147</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>7</v>
       </c>
       <c r="B54" s="4">
-        <f t="shared" si="14"/>
+        <f t="shared" ref="B54:B55" si="14">ROW(A53)</f>
         <v>53</v>
       </c>
       <c r="C54" s="5" t="s">
@@ -2567,12 +2664,12 @@
         <v>149</v>
       </c>
     </row>
-    <row r="55" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>7</v>
       </c>
       <c r="B55" s="4">
-        <f t="shared" ref="B55:B56" si="15">ROW(A54)</f>
+        <f t="shared" si="14"/>
         <v>54</v>
       </c>
       <c r="C55" s="5" t="s">
@@ -2588,12 +2685,12 @@
         <v>151</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>7</v>
       </c>
       <c r="B56" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" ref="B56:B57" si="15">ROW(A55)</f>
         <v>55</v>
       </c>
       <c r="C56" s="5" t="s">
@@ -2609,12 +2706,12 @@
         <v>153</v>
       </c>
     </row>
-    <row r="57" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>7</v>
       </c>
       <c r="B57" s="4">
-        <f t="shared" ref="B57:B58" si="16">ROW(A56)</f>
+        <f t="shared" si="15"/>
         <v>56</v>
       </c>
       <c r="C57" s="5" t="s">
@@ -2630,12 +2727,12 @@
         <v>155</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B58" s="4">
-        <f t="shared" si="16"/>
+        <f t="shared" ref="B58:B59" si="16">ROW(A57)</f>
         <v>57</v>
       </c>
       <c r="C58" s="5" t="s">
@@ -2651,33 +2748,33 @@
         <v>157</v>
       </c>
     </row>
-    <row r="59" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B59" s="4">
-        <f t="shared" ref="B59:B60" si="17">ROW(A58)</f>
+        <f t="shared" si="16"/>
         <v>58</v>
       </c>
       <c r="C59" s="5" t="s">
         <v>55</v>
       </c>
       <c r="D59" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="E59" t="s">
+        <v>28</v>
+      </c>
+      <c r="F59" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="E59" t="s">
-        <v>28</v>
-      </c>
-      <c r="F59" s="1" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="60" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B60" s="4">
-        <f t="shared" si="17"/>
+        <f t="shared" ref="B60:B61" si="17">ROW(A59)</f>
         <v>59</v>
       </c>
       <c r="C60" s="5" t="s">
@@ -2693,12 +2790,12 @@
         <v>161</v>
       </c>
     </row>
-    <row r="61" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B61" s="4">
-        <f t="shared" ref="B61:B62" si="18">ROW(A60)</f>
+        <f t="shared" si="17"/>
         <v>60</v>
       </c>
       <c r="C61" s="5" t="s">
@@ -2714,12 +2811,12 @@
         <v>163</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B62" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" ref="B62:B63" si="18">ROW(A61)</f>
         <v>61</v>
       </c>
       <c r="C62" s="5" t="s">
@@ -2735,12 +2832,12 @@
         <v>165</v>
       </c>
     </row>
-    <row r="63" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B63" s="4">
-        <f t="shared" ref="B63:B64" si="19">ROW(A62)</f>
+        <f t="shared" si="18"/>
         <v>62</v>
       </c>
       <c r="C63" s="5" t="s">
@@ -2756,12 +2853,12 @@
         <v>167</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B64" s="4">
-        <f t="shared" si="19"/>
+        <f t="shared" ref="B64:B65" si="19">ROW(A63)</f>
         <v>63</v>
       </c>
       <c r="C64" s="5" t="s">
@@ -2777,12 +2874,12 @@
         <v>169</v>
       </c>
     </row>
-    <row r="65" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>3</v>
       </c>
       <c r="B65" s="4">
-        <f t="shared" ref="B65:B66" si="20">ROW(A64)</f>
+        <f t="shared" si="19"/>
         <v>64</v>
       </c>
       <c r="C65" s="5" t="s">
@@ -2798,33 +2895,33 @@
         <v>171</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>3</v>
       </c>
       <c r="B66" s="4">
-        <f t="shared" si="20"/>
+        <f t="shared" ref="B66" si="20">ROW(A65)</f>
         <v>65</v>
       </c>
       <c r="C66" s="5" t="s">
         <v>55</v>
       </c>
       <c r="D66" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="E66" t="s">
+        <v>28</v>
+      </c>
+      <c r="F66" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="E66" t="s">
-        <v>28</v>
-      </c>
-      <c r="F66" s="1" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="67" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>3</v>
       </c>
       <c r="B67" s="4">
-        <f t="shared" ref="B67:B68" si="21">ROW(A66)</f>
+        <f t="shared" ref="B67" si="21">ROW(A66)</f>
         <v>66</v>
       </c>
       <c r="C67" s="5" t="s">
@@ -2845,7 +2942,7 @@
         <v>3</v>
       </c>
       <c r="B68" s="4">
-        <f t="shared" si="21"/>
+        <f t="shared" ref="B68" si="22">ROW(A67)</f>
         <v>67</v>
       </c>
       <c r="C68" s="5" t="s">
@@ -2866,7 +2963,7 @@
         <v>3</v>
       </c>
       <c r="B69" s="4">
-        <f t="shared" ref="B69:B70" si="22">ROW(A68)</f>
+        <f t="shared" ref="B69" si="23">ROW(A68)</f>
         <v>68</v>
       </c>
       <c r="C69" s="5" t="s">
@@ -2887,20 +2984,20 @@
         <v>3</v>
       </c>
       <c r="B70" s="4">
-        <f t="shared" si="22"/>
+        <f t="shared" ref="B70" si="24">ROW(A69)</f>
         <v>69</v>
       </c>
       <c r="C70" s="5" t="s">
         <v>55</v>
       </c>
       <c r="D70" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="E70" t="s">
+        <v>28</v>
+      </c>
+      <c r="F70" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="E70" t="s">
-        <v>28</v>
-      </c>
-      <c r="F70" s="1" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="71" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2908,28 +3005,28 @@
         <v>3</v>
       </c>
       <c r="B71" s="4">
-        <f t="shared" ref="B71:B72" si="23">ROW(A70)</f>
+        <f t="shared" ref="B71" si="25">ROW(A70)</f>
         <v>70</v>
       </c>
       <c r="C71" s="5" t="s">
         <v>55</v>
       </c>
       <c r="D71" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="E71" t="s">
+        <v>28</v>
+      </c>
+      <c r="F71" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="E71" t="s">
-        <v>28</v>
-      </c>
-      <c r="F71" s="1" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="72" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>3</v>
       </c>
       <c r="B72" s="4">
-        <f t="shared" si="23"/>
+        <f t="shared" ref="B72" si="26">ROW(A71)</f>
         <v>71</v>
       </c>
       <c r="C72" s="5" t="s">
@@ -2950,7 +3047,7 @@
         <v>3</v>
       </c>
       <c r="B73" s="4">
-        <f t="shared" ref="B73" si="24">ROW(A72)</f>
+        <f t="shared" ref="B73" si="27">ROW(A72)</f>
         <v>72</v>
       </c>
       <c r="C73" s="5" t="s">
@@ -2971,7 +3068,7 @@
         <v>3</v>
       </c>
       <c r="B74" s="4">
-        <f t="shared" ref="B74" si="25">ROW(A73)</f>
+        <f t="shared" ref="B74" si="28">ROW(A73)</f>
         <v>73</v>
       </c>
       <c r="C74" s="5" t="s">
@@ -2992,7 +3089,7 @@
         <v>3</v>
       </c>
       <c r="B75" s="4">
-        <f t="shared" ref="B75" si="26">ROW(A74)</f>
+        <f t="shared" ref="B75" si="29">ROW(A74)</f>
         <v>74</v>
       </c>
       <c r="C75" s="5" t="s">
@@ -3013,7 +3110,7 @@
         <v>3</v>
       </c>
       <c r="B76" s="4">
-        <f t="shared" ref="B76" si="27">ROW(A75)</f>
+        <f t="shared" ref="B76" si="30">ROW(A75)</f>
         <v>75</v>
       </c>
       <c r="C76" s="5" t="s">
@@ -3034,20 +3131,20 @@
         <v>3</v>
       </c>
       <c r="B77" s="4">
-        <f t="shared" ref="B77" si="28">ROW(A76)</f>
+        <f t="shared" ref="B77" si="31">ROW(A76)</f>
         <v>76</v>
       </c>
       <c r="C77" s="5" t="s">
         <v>55</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E77" t="s">
         <v>28</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="78" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3055,28 +3152,28 @@
         <v>3</v>
       </c>
       <c r="B78" s="4">
-        <f t="shared" ref="B78" si="29">ROW(A77)</f>
+        <f t="shared" ref="B78" si="32">ROW(A77)</f>
         <v>77</v>
       </c>
       <c r="C78" s="5" t="s">
         <v>55</v>
       </c>
       <c r="D78" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E78" t="s">
         <v>28</v>
       </c>
       <c r="F78" s="1" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>3</v>
       </c>
       <c r="B79" s="4">
-        <f t="shared" ref="B79" si="30">ROW(A78)</f>
+        <f t="shared" ref="B79" si="33">ROW(A78)</f>
         <v>78</v>
       </c>
       <c r="C79" s="5" t="s">
@@ -3092,12 +3189,12 @@
         <v>199</v>
       </c>
     </row>
-    <row r="80" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>3</v>
       </c>
       <c r="B80" s="4">
-        <f t="shared" ref="B80" si="31">ROW(A79)</f>
+        <f t="shared" ref="B80" si="34">ROW(A79)</f>
         <v>79</v>
       </c>
       <c r="C80" s="5" t="s">
@@ -3113,12 +3210,12 @@
         <v>201</v>
       </c>
     </row>
-    <row r="81" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>3</v>
       </c>
       <c r="B81" s="4">
-        <f t="shared" ref="B81" si="32">ROW(A80)</f>
+        <f t="shared" ref="B81" si="35">ROW(A80)</f>
         <v>80</v>
       </c>
       <c r="C81" s="5" t="s">
@@ -3134,12 +3231,12 @@
         <v>203</v>
       </c>
     </row>
-    <row r="82" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>3</v>
       </c>
       <c r="B82" s="4">
-        <f t="shared" ref="B82" si="33">ROW(A81)</f>
+        <f t="shared" ref="B82" si="36">ROW(A81)</f>
         <v>81</v>
       </c>
       <c r="C82" s="5" t="s">
@@ -3155,12 +3252,12 @@
         <v>205</v>
       </c>
     </row>
-    <row r="83" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>3</v>
       </c>
       <c r="B83" s="4">
-        <f t="shared" ref="B83" si="34">ROW(A82)</f>
+        <f t="shared" ref="B83" si="37">ROW(A82)</f>
         <v>82</v>
       </c>
       <c r="C83" s="5" t="s">
@@ -3176,12 +3273,12 @@
         <v>207</v>
       </c>
     </row>
-    <row r="84" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>3</v>
       </c>
       <c r="B84" s="4">
-        <f t="shared" ref="B84" si="35">ROW(A83)</f>
+        <f t="shared" ref="B84" si="38">ROW(A83)</f>
         <v>83</v>
       </c>
       <c r="C84" s="5" t="s">
@@ -3197,12 +3294,12 @@
         <v>209</v>
       </c>
     </row>
-    <row r="85" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>3</v>
       </c>
       <c r="B85" s="4">
-        <f t="shared" ref="B85" si="36">ROW(A84)</f>
+        <f t="shared" ref="B85" si="39">ROW(A84)</f>
         <v>84</v>
       </c>
       <c r="C85" s="5" t="s">
@@ -3223,7 +3320,7 @@
         <v>3</v>
       </c>
       <c r="B86" s="4">
-        <f t="shared" ref="B86" si="37">ROW(A85)</f>
+        <f t="shared" ref="B86" si="40">ROW(A85)</f>
         <v>85</v>
       </c>
       <c r="C86" s="5" t="s">
@@ -3244,7 +3341,7 @@
         <v>3</v>
       </c>
       <c r="B87" s="4">
-        <f t="shared" ref="B87" si="38">ROW(A86)</f>
+        <f t="shared" ref="B87" si="41">ROW(A86)</f>
         <v>86</v>
       </c>
       <c r="C87" s="5" t="s">
@@ -3265,7 +3362,7 @@
         <v>3</v>
       </c>
       <c r="B88" s="4">
-        <f t="shared" ref="B88" si="39">ROW(A87)</f>
+        <f t="shared" ref="B88" si="42">ROW(A87)</f>
         <v>87</v>
       </c>
       <c r="C88" s="5" t="s">
@@ -3286,7 +3383,7 @@
         <v>3</v>
       </c>
       <c r="B89" s="4">
-        <f t="shared" ref="B89" si="40">ROW(A88)</f>
+        <f t="shared" ref="B89" si="43">ROW(A88)</f>
         <v>88</v>
       </c>
       <c r="C89" s="5" t="s">
@@ -3307,7 +3404,7 @@
         <v>3</v>
       </c>
       <c r="B90" s="4">
-        <f t="shared" ref="B90" si="41">ROW(A89)</f>
+        <f t="shared" ref="B90" si="44">ROW(A89)</f>
         <v>89</v>
       </c>
       <c r="C90" s="5" t="s">
@@ -3328,7 +3425,7 @@
         <v>3</v>
       </c>
       <c r="B91" s="4">
-        <f t="shared" ref="B91" si="42">ROW(A90)</f>
+        <f t="shared" ref="B91" si="45">ROW(A90)</f>
         <v>90</v>
       </c>
       <c r="C91" s="5" t="s">
@@ -3349,7 +3446,7 @@
         <v>3</v>
       </c>
       <c r="B92" s="4">
-        <f t="shared" ref="B92" si="43">ROW(A91)</f>
+        <f t="shared" ref="B92" si="46">ROW(A91)</f>
         <v>91</v>
       </c>
       <c r="C92" s="5" t="s">
@@ -3370,7 +3467,7 @@
         <v>3</v>
       </c>
       <c r="B93" s="4">
-        <f t="shared" ref="B93" si="44">ROW(A92)</f>
+        <f t="shared" ref="B93" si="47">ROW(A92)</f>
         <v>92</v>
       </c>
       <c r="C93" s="5" t="s">
@@ -3391,7 +3488,7 @@
         <v>3</v>
       </c>
       <c r="B94" s="4">
-        <f t="shared" ref="B94" si="45">ROW(A93)</f>
+        <f t="shared" ref="B94" si="48">ROW(A93)</f>
         <v>93</v>
       </c>
       <c r="C94" s="5" t="s">
@@ -3412,7 +3509,7 @@
         <v>3</v>
       </c>
       <c r="B95" s="4">
-        <f t="shared" ref="B95" si="46">ROW(A94)</f>
+        <f t="shared" ref="B95" si="49">ROW(A94)</f>
         <v>94</v>
       </c>
       <c r="C95" s="5" t="s">
@@ -3433,7 +3530,7 @@
         <v>3</v>
       </c>
       <c r="B96" s="4">
-        <f t="shared" ref="B96" si="47">ROW(A95)</f>
+        <f t="shared" ref="B96" si="50">ROW(A95)</f>
         <v>95</v>
       </c>
       <c r="C96" s="5" t="s">
@@ -3454,7 +3551,7 @@
         <v>3</v>
       </c>
       <c r="B97" s="4">
-        <f t="shared" ref="B97" si="48">ROW(A96)</f>
+        <f t="shared" ref="B97" si="51">ROW(A96)</f>
         <v>96</v>
       </c>
       <c r="C97" s="5" t="s">
@@ -3475,7 +3572,7 @@
         <v>3</v>
       </c>
       <c r="B98" s="4">
-        <f t="shared" ref="B98" si="49">ROW(A97)</f>
+        <f t="shared" ref="B98" si="52">ROW(A97)</f>
         <v>97</v>
       </c>
       <c r="C98" s="5" t="s">
@@ -3496,7 +3593,7 @@
         <v>3</v>
       </c>
       <c r="B99" s="4">
-        <f t="shared" ref="B99" si="50">ROW(A98)</f>
+        <f t="shared" ref="B99" si="53">ROW(A98)</f>
         <v>98</v>
       </c>
       <c r="C99" s="5" t="s">
@@ -3517,7 +3614,7 @@
         <v>3</v>
       </c>
       <c r="B100" s="4">
-        <f t="shared" ref="B100" si="51">ROW(A99)</f>
+        <f t="shared" ref="B100" si="54">ROW(A99)</f>
         <v>99</v>
       </c>
       <c r="C100" s="5" t="s">
@@ -3538,7 +3635,7 @@
         <v>3</v>
       </c>
       <c r="B101" s="4">
-        <f t="shared" ref="B101" si="52">ROW(A100)</f>
+        <f t="shared" ref="B101" si="55">ROW(A100)</f>
         <v>100</v>
       </c>
       <c r="C101" s="5" t="s">
@@ -3559,7 +3656,7 @@
         <v>3</v>
       </c>
       <c r="B102" s="4">
-        <f t="shared" ref="B102" si="53">ROW(A101)</f>
+        <f t="shared" ref="B102" si="56">ROW(A101)</f>
         <v>101</v>
       </c>
       <c r="C102" s="5" t="s">
@@ -3580,7 +3677,7 @@
         <v>3</v>
       </c>
       <c r="B103" s="4">
-        <f t="shared" ref="B103" si="54">ROW(A102)</f>
+        <f t="shared" ref="B103" si="57">ROW(A102)</f>
         <v>102</v>
       </c>
       <c r="C103" s="5" t="s">
@@ -3601,7 +3698,7 @@
         <v>3</v>
       </c>
       <c r="B104" s="4">
-        <f t="shared" ref="B104" si="55">ROW(A103)</f>
+        <f t="shared" ref="B104" si="58">ROW(A103)</f>
         <v>103</v>
       </c>
       <c r="C104" s="5" t="s">
@@ -3622,7 +3719,7 @@
         <v>3</v>
       </c>
       <c r="B105" s="4">
-        <f t="shared" ref="B105" si="56">ROW(A104)</f>
+        <f t="shared" ref="B105" si="59">ROW(A104)</f>
         <v>104</v>
       </c>
       <c r="C105" s="5" t="s">
@@ -3643,7 +3740,7 @@
         <v>3</v>
       </c>
       <c r="B106" s="4">
-        <f t="shared" ref="B106" si="57">ROW(A105)</f>
+        <f t="shared" ref="B106" si="60">ROW(A105)</f>
         <v>105</v>
       </c>
       <c r="C106" s="5" t="s">
@@ -3664,7 +3761,7 @@
         <v>3</v>
       </c>
       <c r="B107" s="4">
-        <f t="shared" ref="B107" si="58">ROW(A106)</f>
+        <f t="shared" ref="B107" si="61">ROW(A106)</f>
         <v>106</v>
       </c>
       <c r="C107" s="5" t="s">
@@ -3685,7 +3782,7 @@
         <v>3</v>
       </c>
       <c r="B108" s="4">
-        <f t="shared" ref="B108" si="59">ROW(A107)</f>
+        <f t="shared" ref="B108" si="62">ROW(A107)</f>
         <v>107</v>
       </c>
       <c r="C108" s="5" t="s">
@@ -3706,7 +3803,7 @@
         <v>3</v>
       </c>
       <c r="B109" s="4">
-        <f t="shared" ref="B109" si="60">ROW(A108)</f>
+        <f t="shared" ref="B109" si="63">ROW(A108)</f>
         <v>108</v>
       </c>
       <c r="C109" s="5" t="s">
@@ -3727,7 +3824,7 @@
         <v>3</v>
       </c>
       <c r="B110" s="4">
-        <f t="shared" ref="B110" si="61">ROW(A109)</f>
+        <f t="shared" ref="B110" si="64">ROW(A109)</f>
         <v>109</v>
       </c>
       <c r="C110" s="5" t="s">
@@ -3748,7 +3845,7 @@
         <v>3</v>
       </c>
       <c r="B111" s="4">
-        <f t="shared" ref="B111" si="62">ROW(A110)</f>
+        <f t="shared" ref="B111" si="65">ROW(A110)</f>
         <v>110</v>
       </c>
       <c r="C111" s="5" t="s">
@@ -3769,20 +3866,20 @@
         <v>3</v>
       </c>
       <c r="B112" s="4">
-        <f t="shared" ref="B112" si="63">ROW(A111)</f>
+        <f t="shared" ref="B112" si="66">ROW(A111)</f>
         <v>111</v>
       </c>
       <c r="C112" s="5" t="s">
         <v>55</v>
       </c>
       <c r="D112" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="E112" t="s">
+        <v>28</v>
+      </c>
+      <c r="F112" s="1" t="s">
         <v>264</v>
-      </c>
-      <c r="E112" t="s">
-        <v>28</v>
-      </c>
-      <c r="F112" s="1" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="113" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3790,7 +3887,7 @@
         <v>3</v>
       </c>
       <c r="B113" s="4">
-        <f t="shared" ref="B113" si="64">ROW(A112)</f>
+        <f t="shared" ref="B113" si="67">ROW(A112)</f>
         <v>112</v>
       </c>
       <c r="C113" s="5" t="s">
@@ -3811,7 +3908,7 @@
         <v>3</v>
       </c>
       <c r="B114" s="4">
-        <f t="shared" ref="B114" si="65">ROW(A113)</f>
+        <f t="shared" ref="B114" si="68">ROW(A113)</f>
         <v>113</v>
       </c>
       <c r="C114" s="5" t="s">
@@ -3832,7 +3929,7 @@
         <v>3</v>
       </c>
       <c r="B115" s="4">
-        <f t="shared" ref="B115" si="66">ROW(A114)</f>
+        <f t="shared" ref="B115" si="69">ROW(A114)</f>
         <v>114</v>
       </c>
       <c r="C115" s="5" t="s">
@@ -3853,7 +3950,7 @@
         <v>3</v>
       </c>
       <c r="B116" s="4">
-        <f t="shared" ref="B116" si="67">ROW(A115)</f>
+        <f t="shared" ref="B116" si="70">ROW(A115)</f>
         <v>115</v>
       </c>
       <c r="C116" s="5" t="s">
@@ -3874,7 +3971,7 @@
         <v>3</v>
       </c>
       <c r="B117" s="4">
-        <f t="shared" ref="B117" si="68">ROW(A116)</f>
+        <f t="shared" ref="B117" si="71">ROW(A116)</f>
         <v>116</v>
       </c>
       <c r="C117" s="5" t="s">
@@ -3895,20 +3992,20 @@
         <v>3</v>
       </c>
       <c r="B118" s="4">
-        <f t="shared" ref="B118" si="69">ROW(A117)</f>
+        <f t="shared" ref="B118" si="72">ROW(A117)</f>
         <v>117</v>
       </c>
       <c r="C118" s="5" t="s">
         <v>55</v>
       </c>
       <c r="D118" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="E118" t="s">
+        <v>28</v>
+      </c>
+      <c r="F118" s="1" t="s">
         <v>276</v>
-      </c>
-      <c r="E118" t="s">
-        <v>28</v>
-      </c>
-      <c r="F118" s="1" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="119" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3916,20 +4013,20 @@
         <v>3</v>
       </c>
       <c r="B119" s="4">
-        <f t="shared" ref="B119" si="70">ROW(A118)</f>
+        <f t="shared" ref="B119" si="73">ROW(A118)</f>
         <v>118</v>
       </c>
       <c r="C119" s="5" t="s">
         <v>55</v>
       </c>
       <c r="D119" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="E119" t="s">
+        <v>28</v>
+      </c>
+      <c r="F119" s="1" t="s">
         <v>279</v>
-      </c>
-      <c r="E119" t="s">
-        <v>28</v>
-      </c>
-      <c r="F119" s="1" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="120" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3937,7 +4034,7 @@
         <v>3</v>
       </c>
       <c r="B120" s="4">
-        <f t="shared" ref="B120" si="71">ROW(A119)</f>
+        <f t="shared" ref="B120" si="74">ROW(A119)</f>
         <v>119</v>
       </c>
       <c r="C120" s="5" t="s">
@@ -3958,7 +4055,7 @@
         <v>3</v>
       </c>
       <c r="B121" s="4">
-        <f t="shared" ref="B121" si="72">ROW(A120)</f>
+        <f t="shared" ref="B121" si="75">ROW(A120)</f>
         <v>120</v>
       </c>
       <c r="C121" s="5" t="s">
@@ -3979,7 +4076,7 @@
         <v>3</v>
       </c>
       <c r="B122" s="4">
-        <f t="shared" ref="B122" si="73">ROW(A121)</f>
+        <f t="shared" ref="B122" si="76">ROW(A121)</f>
         <v>121</v>
       </c>
       <c r="C122" s="5" t="s">
@@ -4000,7 +4097,7 @@
         <v>3</v>
       </c>
       <c r="B123" s="4">
-        <f t="shared" ref="B123" si="74">ROW(A122)</f>
+        <f t="shared" ref="B123" si="77">ROW(A122)</f>
         <v>122</v>
       </c>
       <c r="C123" s="5" t="s">
@@ -4021,7 +4118,7 @@
         <v>3</v>
       </c>
       <c r="B124" s="4">
-        <f t="shared" ref="B124" si="75">ROW(A123)</f>
+        <f t="shared" ref="B124" si="78">ROW(A123)</f>
         <v>123</v>
       </c>
       <c r="C124" s="5" t="s">
@@ -4039,31 +4136,31 @@
     </row>
     <row r="125" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B125" s="4">
-        <f t="shared" ref="B125" si="76">ROW(A124)</f>
+        <f t="shared" ref="B125" si="79">ROW(A124)</f>
         <v>124</v>
       </c>
       <c r="C125" s="5" t="s">
         <v>55</v>
       </c>
       <c r="D125" s="5" t="s">
+        <v>290</v>
+      </c>
+      <c r="E125" t="s">
+        <v>28</v>
+      </c>
+      <c r="F125" s="1" t="s">
         <v>291</v>
-      </c>
-      <c r="E125" t="s">
-        <v>28</v>
-      </c>
-      <c r="F125" s="1" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="126" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B126" s="4">
-        <f t="shared" ref="B126" si="77">ROW(A125)</f>
+        <f t="shared" ref="B126" si="80">ROW(A125)</f>
         <v>125</v>
       </c>
       <c r="C126" s="5" t="s">
@@ -4081,10 +4178,10 @@
     </row>
     <row r="127" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B127" s="4">
-        <f t="shared" ref="B127" si="78">ROW(A126)</f>
+        <f t="shared" ref="B127" si="81">ROW(A126)</f>
         <v>126</v>
       </c>
       <c r="C127" s="5" t="s">
@@ -4102,10 +4199,10 @@
     </row>
     <row r="128" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B128" s="4">
-        <f t="shared" ref="B128" si="79">ROW(A127)</f>
+        <f t="shared" ref="B128" si="82">ROW(A127)</f>
         <v>127</v>
       </c>
       <c r="C128" s="5" t="s">
@@ -4121,12 +4218,12 @@
         <v>297</v>
       </c>
     </row>
-    <row r="129" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B129" s="4">
-        <f t="shared" ref="B129" si="80">ROW(A128)</f>
+        <f t="shared" ref="B129" si="83">ROW(A128)</f>
         <v>128</v>
       </c>
       <c r="C129" s="5" t="s">
@@ -4142,12 +4239,12 @@
         <v>299</v>
       </c>
     </row>
-    <row r="130" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B130" s="4">
-        <f t="shared" ref="B130" si="81">ROW(A129)</f>
+        <f t="shared" ref="B130" si="84">ROW(A129)</f>
         <v>129</v>
       </c>
       <c r="C130" s="5" t="s">
@@ -4163,12 +4260,12 @@
         <v>301</v>
       </c>
     </row>
-    <row r="131" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B131" s="4">
-        <f t="shared" ref="B131" si="82">ROW(A130)</f>
+        <f t="shared" ref="B131" si="85">ROW(A130)</f>
         <v>130</v>
       </c>
       <c r="C131" s="5" t="s">
@@ -4184,12 +4281,12 @@
         <v>303</v>
       </c>
     </row>
-    <row r="132" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>7</v>
       </c>
       <c r="B132" s="4">
-        <f t="shared" ref="B132" si="83">ROW(A131)</f>
+        <f t="shared" ref="B132" si="86">ROW(A131)</f>
         <v>131</v>
       </c>
       <c r="C132" s="5" t="s">
@@ -4205,12 +4302,12 @@
         <v>305</v>
       </c>
     </row>
-    <row r="133" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>7</v>
       </c>
       <c r="B133" s="4">
-        <f t="shared" ref="B133" si="84">ROW(A132)</f>
+        <f t="shared" ref="B133" si="87">ROW(A132)</f>
         <v>132</v>
       </c>
       <c r="C133" s="5" t="s">
@@ -4226,12 +4323,12 @@
         <v>307</v>
       </c>
     </row>
-    <row r="134" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>7</v>
       </c>
       <c r="B134" s="4">
-        <f t="shared" ref="B134" si="85">ROW(A133)</f>
+        <f t="shared" ref="B134" si="88">ROW(A133)</f>
         <v>133</v>
       </c>
       <c r="C134" s="5" t="s">
@@ -4247,12 +4344,12 @@
         <v>309</v>
       </c>
     </row>
-    <row r="135" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>7</v>
       </c>
       <c r="B135" s="4">
-        <f t="shared" ref="B135" si="86">ROW(A134)</f>
+        <f t="shared" ref="B135" si="89">ROW(A134)</f>
         <v>134</v>
       </c>
       <c r="C135" s="5" t="s">
@@ -4268,158 +4365,398 @@
         <v>311</v>
       </c>
     </row>
-    <row r="136" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A136" t="s">
-        <v>7</v>
-      </c>
-      <c r="B136" s="4">
-        <f t="shared" ref="B136" si="87">ROW(A135)</f>
+    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A136" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B136" s="7">
         <v>135</v>
       </c>
-      <c r="C136" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D136" s="5" t="s">
+      <c r="C136" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D136" s="8" t="s">
         <v>312</v>
       </c>
-      <c r="E136" t="s">
-        <v>28</v>
-      </c>
-      <c r="F136" s="1" t="s">
+      <c r="E136" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F136" s="10" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="137" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A137" t="s">
-        <v>7</v>
-      </c>
-      <c r="B137" s="4">
-        <f t="shared" ref="B137" si="88">ROW(A136)</f>
+      <c r="G136" s="6"/>
+      <c r="H136" s="7"/>
+      <c r="I136" s="8"/>
+      <c r="J136" s="8"/>
+    </row>
+    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A137" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B137" s="7">
         <v>136</v>
       </c>
-      <c r="C137" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D137" s="5" t="s">
+      <c r="C137" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D137" s="8" t="s">
         <v>314</v>
       </c>
-      <c r="E137" t="s">
-        <v>28</v>
-      </c>
-      <c r="F137" s="1" t="s">
+      <c r="E137" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F137" s="10" t="s">
         <v>315</v>
       </c>
-    </row>
-    <row r="138" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A138" t="s">
-        <v>7</v>
-      </c>
-      <c r="B138" s="4">
-        <f t="shared" ref="B138" si="89">ROW(A137)</f>
+      <c r="G137" s="6"/>
+      <c r="H137" s="7"/>
+      <c r="I137" s="8"/>
+      <c r="J137" s="8"/>
+    </row>
+    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A138" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B138" s="7">
         <v>137</v>
       </c>
-      <c r="C138" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D138" s="5" t="s">
+      <c r="C138" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D138" s="8" t="s">
         <v>316</v>
       </c>
-      <c r="E138" t="s">
-        <v>28</v>
-      </c>
-      <c r="F138" s="1" t="s">
+      <c r="E138" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F138" s="10" t="s">
         <v>317</v>
       </c>
-    </row>
-    <row r="139" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A139" t="s">
-        <v>7</v>
-      </c>
-      <c r="B139" s="4">
-        <f t="shared" ref="B139" si="90">ROW(A138)</f>
+      <c r="G138" s="6"/>
+      <c r="H138" s="7"/>
+      <c r="I138" s="8"/>
+      <c r="J138" s="8"/>
+    </row>
+    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A139" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B139" s="7">
         <v>138</v>
       </c>
-      <c r="C139" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D139" s="5" t="s">
+      <c r="C139" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D139" s="8" t="s">
         <v>318</v>
       </c>
-      <c r="E139" t="s">
-        <v>28</v>
-      </c>
-      <c r="F139" s="1" t="s">
+      <c r="E139" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F139" s="10" t="s">
         <v>319</v>
       </c>
-    </row>
-    <row r="140" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A140" t="s">
-        <v>7</v>
-      </c>
-      <c r="B140" s="4">
-        <f t="shared" ref="B140" si="91">ROW(A139)</f>
+      <c r="G139" s="6"/>
+      <c r="H139" s="7"/>
+      <c r="I139" s="8"/>
+      <c r="J139" s="8"/>
+    </row>
+    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A140" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B140" s="7">
         <v>139</v>
       </c>
-      <c r="C140" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D140" s="5" t="s">
+      <c r="C140" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D140" s="8" t="s">
         <v>320</v>
       </c>
-      <c r="E140" t="s">
-        <v>28</v>
-      </c>
-      <c r="F140" s="1" t="s">
+      <c r="E140" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F140" s="10" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="141" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A141" t="s">
-        <v>7</v>
-      </c>
-      <c r="B141" s="4">
-        <f t="shared" ref="B141" si="92">ROW(A140)</f>
+      <c r="G140" s="6"/>
+      <c r="H140" s="7"/>
+      <c r="I140" s="8"/>
+      <c r="J140" s="8"/>
+    </row>
+    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A141" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B141" s="7">
         <v>140</v>
       </c>
-      <c r="C141" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D141" s="5" t="s">
+      <c r="C141" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D141" s="8" t="s">
         <v>322</v>
       </c>
-      <c r="E141" t="s">
-        <v>28</v>
-      </c>
-      <c r="F141" s="1" t="s">
+      <c r="E141" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F141" s="10" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="142" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A142" t="s">
-        <v>7</v>
-      </c>
-      <c r="B142" s="4">
-        <f t="shared" ref="B142" si="93">ROW(A141)</f>
+      <c r="G141" s="6"/>
+      <c r="H141" s="7"/>
+      <c r="I141" s="8"/>
+      <c r="J141" s="8"/>
+    </row>
+    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A142" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B142" s="7">
         <v>141</v>
       </c>
-      <c r="C142" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D142" s="5" t="s">
+      <c r="C142" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D142" s="8" t="s">
         <v>324</v>
       </c>
-      <c r="E142" t="s">
-        <v>28</v>
-      </c>
-      <c r="F142" s="1" t="s">
+      <c r="E142" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F142" s="10" t="s">
         <v>325</v>
       </c>
+      <c r="G142" s="6"/>
+      <c r="H142" s="7"/>
+      <c r="I142" s="8"/>
+      <c r="J142" s="8"/>
+    </row>
+    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A143" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B143" s="7">
+        <v>142</v>
+      </c>
+      <c r="C143" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D143" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="E143" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F143" s="10" t="s">
+        <v>327</v>
+      </c>
+      <c r="G143" s="6"/>
+      <c r="H143" s="7"/>
+      <c r="I143" s="8"/>
+      <c r="J143" s="8"/>
+    </row>
+    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A144" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B144" s="7">
+        <v>143</v>
+      </c>
+      <c r="C144" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D144" s="8" t="s">
+        <v>328</v>
+      </c>
+      <c r="E144" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F144" s="10" t="s">
+        <v>329</v>
+      </c>
+      <c r="G144" s="6"/>
+      <c r="H144" s="7"/>
+      <c r="I144" s="8"/>
+      <c r="J144" s="8"/>
+    </row>
+    <row r="145" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A145" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B145" s="7">
+        <v>144</v>
+      </c>
+      <c r="C145" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D145" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="E145" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F145" s="10" t="s">
+        <v>331</v>
+      </c>
+      <c r="G145" s="6"/>
+      <c r="H145" s="7"/>
+      <c r="I145" s="8"/>
+      <c r="J145" s="8"/>
+    </row>
+    <row r="146" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A146" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B146" s="7">
+        <v>145</v>
+      </c>
+      <c r="C146" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D146" s="8" t="s">
+        <v>332</v>
+      </c>
+      <c r="E146" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F146" s="10" t="s">
+        <v>333</v>
+      </c>
+      <c r="G146" s="6"/>
+      <c r="H146" s="7"/>
+      <c r="I146" s="8"/>
+      <c r="J146" s="8"/>
+    </row>
+    <row r="147" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A147" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B147" s="7">
+        <v>146</v>
+      </c>
+      <c r="C147" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D147" s="8" t="s">
+        <v>334</v>
+      </c>
+      <c r="E147" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F147" s="10" t="s">
+        <v>335</v>
+      </c>
+      <c r="G147" s="6"/>
+      <c r="H147" s="7"/>
+      <c r="I147" s="8"/>
+      <c r="J147" s="8"/>
+    </row>
+    <row r="148" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A148" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B148" s="7">
+        <v>147</v>
+      </c>
+      <c r="C148" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D148" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="E148" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F148" s="10" t="s">
+        <v>337</v>
+      </c>
+      <c r="G148" s="6"/>
+      <c r="H148" s="7"/>
+      <c r="I148" s="8"/>
+      <c r="J148" s="8"/>
+    </row>
+    <row r="149" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A149" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B149" s="7">
+        <v>148</v>
+      </c>
+      <c r="C149" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D149" s="8" t="s">
+        <v>338</v>
+      </c>
+      <c r="E149" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F149" s="10" t="s">
+        <v>339</v>
+      </c>
+      <c r="G149" s="6"/>
+      <c r="H149" s="7"/>
+      <c r="I149" s="8"/>
+      <c r="J149" s="8"/>
+    </row>
+    <row r="150" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A150" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B150" s="7">
+        <v>149</v>
+      </c>
+      <c r="C150" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D150" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="E150" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F150" s="10" t="s">
+        <v>341</v>
+      </c>
+      <c r="G150" s="6"/>
+      <c r="H150" s="7"/>
+      <c r="I150" s="8"/>
+      <c r="J150" s="8"/>
+    </row>
+    <row r="151" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A151" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B151" s="7">
+        <v>150</v>
+      </c>
+      <c r="C151" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D151" s="8" t="s">
+        <v>342</v>
+      </c>
+      <c r="E151" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F151" s="10" t="s">
+        <v>343</v>
+      </c>
+      <c r="G151" s="6"/>
+      <c r="H151" s="7"/>
+      <c r="I151" s="8"/>
+      <c r="J151" s="8"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F26" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -4428,25 +4765,25 @@
           <x14:formula1>
             <xm:f>dpt_delta!$A$2:$A$24</xm:f>
           </x14:formula1>
-          <xm:sqref>A145:A166</xm:sqref>
+          <xm:sqref>A138:A159</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Código de la dpt de parroquia" prompt="Código de la dpt de parroquia">
           <x14:formula1>
             <xm:f>dpt_delta!$A$2:$A$24</xm:f>
           </x14:formula1>
-          <xm:sqref>A143:A144 A1</xm:sqref>
+          <xm:sqref>A136:A137 A1</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>dpt_delta!$B$2:$B$24</xm:f>
           </x14:formula1>
-          <xm:sqref>A2:A142</xm:sqref>
+          <xm:sqref>A2:A135</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Formato de la Publicación" prompt="Formato de la Publicación">
           <x14:formula1>
             <xm:f>formato!$A$2:$A$12</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E142</xm:sqref>
+          <xm:sqref>E2:E135</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Se agregó Francisco Aniceto Lugo
</commit_message>
<xml_diff>
--- a/libro_publicaciones.xlsx
+++ b/libro_publicaciones.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fguedez\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fguedez\Documents\Proyectos\page-estadisticas\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="798" uniqueCount="344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="893" uniqueCount="381">
   <si>
     <t>codigo</t>
   </si>
@@ -1059,6 +1059,117 @@
   </si>
   <si>
     <t>https://drive.google.com/file/d/1Qe2iUdgGKJjrVDY1_0Cx7b4Gec0H0N1R/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  JUANA AJÁ</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1YMiwZ9G6euUMlSilqU5DqKj4jFQmQBBp/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  BUROBAKA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1AYGSZYG7qUPHwyW8-VEJjleyXMJ6y1id/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  MUKOBOINA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1P13Gc4YLb38SJ0w8X1rprzVgOx38U3ji/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  PUNTA BARIMA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1jjX36VXnRT9ZOQ5XL6Frqqhb-QjBB5JC/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  JOMONI</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/12eSCagSvsqwDlFH6EK6yJvzFiwbA62P1/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  MIANARINA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1749TBOg8gtKd5ai75gKQg0vKoGKiWDSZ/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  MEJOKOBOINA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/157Tp8_Dg6qSxuyyy8xqZDMy-sFvaDf1h/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  JANABASA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1_yigwUucF_CpckgMXCoqdOyPHxVQ4jPn/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  BOCA DE AMACURO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1ThKuyLMmtAUMsueLVqUFAv2jQLkwhsgR/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  AUTIAJANA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1iepwTJUg8w3YTF6DKNuso67dMEG8eGuv/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  YORIJEKENUKA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1VQ8DLbHzliPZnuDL7-X-EokWrBJCwSgi/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  LA LINEA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/15RJzMDPqf13SW3tBNdC-DKj8C2pL-Khz/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1gtc1tkyrk61JJemWajD6BCiWO8xx4GfH/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  YARONANOKO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1tuLs9knpJZQcQ-dbkdEOXObD1NLtrGvc/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  EL FARITO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1qMdIuEfgZfn9BBsjp-xcF2Cp0TQ0q47B/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  MORUINA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1yxfSRRE1fya3Pt6TzGpEyPH5E5KyjggD/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  MUJOKOINA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1Zf_Ssc4FZtd8AdfUYMRZ1_AKBRo6cfVG/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  WAYAKAIKORO</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1dUg6aXegRJ5QeAVeHM4qIYNfLiGtGh7E/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  JANATOROSANUKA</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1cJdMNeScb1eGkj4Yipk9Lp7C8wAucJOb/view?usp=drive_link</t>
   </si>
 </sst>
 </file>
@@ -1521,7 +1632,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J151"/>
+  <dimension ref="A1:J170"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -4748,6 +4859,405 @@
       <c r="H151" s="7"/>
       <c r="I151" s="8"/>
       <c r="J151" s="8"/>
+    </row>
+    <row r="152" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>5</v>
+      </c>
+      <c r="B152" s="4">
+        <f t="shared" ref="B152" si="90">ROW(A151)</f>
+        <v>151</v>
+      </c>
+      <c r="C152" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D152" s="5" t="s">
+        <v>344</v>
+      </c>
+      <c r="E152" t="s">
+        <v>28</v>
+      </c>
+      <c r="F152" s="1" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="153" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>5</v>
+      </c>
+      <c r="B153" s="4">
+        <f t="shared" ref="B153" si="91">ROW(A152)</f>
+        <v>152</v>
+      </c>
+      <c r="C153" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D153" s="5" t="s">
+        <v>346</v>
+      </c>
+      <c r="E153" t="s">
+        <v>28</v>
+      </c>
+      <c r="F153" s="1" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="154" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>5</v>
+      </c>
+      <c r="B154" s="4">
+        <f t="shared" ref="B154" si="92">ROW(A153)</f>
+        <v>153</v>
+      </c>
+      <c r="C154" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D154" s="5" t="s">
+        <v>348</v>
+      </c>
+      <c r="E154" t="s">
+        <v>28</v>
+      </c>
+      <c r="F154" s="1" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="155" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>5</v>
+      </c>
+      <c r="B155" s="4">
+        <f t="shared" ref="B155" si="93">ROW(A154)</f>
+        <v>154</v>
+      </c>
+      <c r="C155" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D155" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="E155" t="s">
+        <v>28</v>
+      </c>
+      <c r="F155" s="1" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="156" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>5</v>
+      </c>
+      <c r="B156" s="4">
+        <f t="shared" ref="B156" si="94">ROW(A155)</f>
+        <v>155</v>
+      </c>
+      <c r="C156" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D156" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="E156" t="s">
+        <v>28</v>
+      </c>
+      <c r="F156" s="1" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="157" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>5</v>
+      </c>
+      <c r="B157" s="4">
+        <f t="shared" ref="B157" si="95">ROW(A156)</f>
+        <v>156</v>
+      </c>
+      <c r="C157" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D157" s="5" t="s">
+        <v>354</v>
+      </c>
+      <c r="E157" t="s">
+        <v>28</v>
+      </c>
+      <c r="F157" s="1" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="158" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>5</v>
+      </c>
+      <c r="B158" s="4">
+        <f t="shared" ref="B158" si="96">ROW(A157)</f>
+        <v>157</v>
+      </c>
+      <c r="C158" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D158" s="5" t="s">
+        <v>356</v>
+      </c>
+      <c r="E158" t="s">
+        <v>28</v>
+      </c>
+      <c r="F158" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="159" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>5</v>
+      </c>
+      <c r="B159" s="4">
+        <f t="shared" ref="B159" si="97">ROW(A158)</f>
+        <v>158</v>
+      </c>
+      <c r="C159" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D159" s="5" t="s">
+        <v>358</v>
+      </c>
+      <c r="E159" t="s">
+        <v>28</v>
+      </c>
+      <c r="F159" s="1" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="160" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
+        <v>5</v>
+      </c>
+      <c r="B160" s="4">
+        <f t="shared" ref="B160" si="98">ROW(A159)</f>
+        <v>159</v>
+      </c>
+      <c r="C160" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D160" s="5" t="s">
+        <v>360</v>
+      </c>
+      <c r="E160" t="s">
+        <v>28</v>
+      </c>
+      <c r="F160" s="1" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
+        <v>5</v>
+      </c>
+      <c r="B161" s="4">
+        <f t="shared" ref="B161" si="99">ROW(A160)</f>
+        <v>160</v>
+      </c>
+      <c r="C161" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D161" s="5" t="s">
+        <v>362</v>
+      </c>
+      <c r="E161" t="s">
+        <v>28</v>
+      </c>
+      <c r="F161" s="1" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>5</v>
+      </c>
+      <c r="B162" s="4">
+        <f t="shared" ref="B162" si="100">ROW(A161)</f>
+        <v>161</v>
+      </c>
+      <c r="C162" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D162" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="E162" t="s">
+        <v>28</v>
+      </c>
+      <c r="F162" s="1" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
+        <v>5</v>
+      </c>
+      <c r="B163" s="4">
+        <f t="shared" ref="B163" si="101">ROW(A162)</f>
+        <v>162</v>
+      </c>
+      <c r="C163" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D163" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="E163" t="s">
+        <v>28</v>
+      </c>
+      <c r="F163" s="1" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
+        <v>5</v>
+      </c>
+      <c r="B164" s="4">
+        <f t="shared" ref="B164" si="102">ROW(A163)</f>
+        <v>163</v>
+      </c>
+      <c r="C164" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D164" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="E164" t="s">
+        <v>28</v>
+      </c>
+      <c r="F164" s="1" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>5</v>
+      </c>
+      <c r="B165" s="4">
+        <f t="shared" ref="B165" si="103">ROW(A164)</f>
+        <v>164</v>
+      </c>
+      <c r="C165" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D165" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="E165" t="s">
+        <v>28</v>
+      </c>
+      <c r="F165" s="1" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
+        <v>5</v>
+      </c>
+      <c r="B166" s="4">
+        <f t="shared" ref="B166" si="104">ROW(A165)</f>
+        <v>165</v>
+      </c>
+      <c r="C166" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D166" s="5" t="s">
+        <v>371</v>
+      </c>
+      <c r="E166" t="s">
+        <v>28</v>
+      </c>
+      <c r="F166" s="1" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="167" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
+        <v>5</v>
+      </c>
+      <c r="B167" s="4">
+        <f t="shared" ref="B167" si="105">ROW(A166)</f>
+        <v>166</v>
+      </c>
+      <c r="C167" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D167" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="E167" t="s">
+        <v>28</v>
+      </c>
+      <c r="F167" s="1" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
+        <v>5</v>
+      </c>
+      <c r="B168" s="4">
+        <f t="shared" ref="B168" si="106">ROW(A167)</f>
+        <v>167</v>
+      </c>
+      <c r="C168" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D168" s="5" t="s">
+        <v>375</v>
+      </c>
+      <c r="E168" t="s">
+        <v>28</v>
+      </c>
+      <c r="F168" s="1" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="169" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
+        <v>5</v>
+      </c>
+      <c r="B169" s="4">
+        <f t="shared" ref="B169" si="107">ROW(A168)</f>
+        <v>168</v>
+      </c>
+      <c r="C169" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D169" s="5" t="s">
+        <v>377</v>
+      </c>
+      <c r="E169" t="s">
+        <v>28</v>
+      </c>
+      <c r="F169" s="1" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="170" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
+        <v>5</v>
+      </c>
+      <c r="B170" s="4">
+        <f t="shared" ref="B170" si="108">ROW(A169)</f>
+        <v>169</v>
+      </c>
+      <c r="C170" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D170" s="5" t="s">
+        <v>379</v>
+      </c>
+      <c r="E170" t="s">
+        <v>28</v>
+      </c>
+      <c r="F170" s="1" t="s">
+        <v>380</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -4765,7 +5275,7 @@
           <x14:formula1>
             <xm:f>dpt_delta!$A$2:$A$24</xm:f>
           </x14:formula1>
-          <xm:sqref>A138:A159</xm:sqref>
+          <xm:sqref>A138:A151</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Código de la dpt de parroquia" prompt="Código de la dpt de parroquia">
           <x14:formula1>
@@ -4777,13 +5287,13 @@
           <x14:formula1>
             <xm:f>dpt_delta!$B$2:$B$24</xm:f>
           </x14:formula1>
-          <xm:sqref>A2:A135</xm:sqref>
+          <xm:sqref>A2:A135 A152:A170</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Formato de la Publicación" prompt="Formato de la Publicación">
           <x14:formula1>
             <xm:f>formato!$A$2:$A$12</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E135</xm:sqref>
+          <xm:sqref>E2:E135 E152:E170</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Se agregó microareas  urbanas
</commit_message>
<xml_diff>
--- a/libro_publicaciones.xlsx
+++ b/libro_publicaciones.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="893" uniqueCount="381">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="945" uniqueCount="402">
   <si>
     <t>codigo</t>
   </si>
@@ -1170,6 +1170,69 @@
   </si>
   <si>
     <t>https://drive.google.com/file/d/1cJdMNeScb1eGkj4Yipk9Lp7C8wAucJOb/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>Microareas Urbanas Parroquia Argimiro García</t>
+  </si>
+  <si>
+    <t>Microarea Urbana Censo 2011</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/presentation/d/1BXo1Lf48G3eZvivzMTuU4A8GP4mwpU3W/edit?usp=drive_link&amp;ouid=105142876406402750370&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>Microareas Urbanas Parroquia Virgen del Valle</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/presentation/d/13whKTEo8OlCT0PgBrLIH6reIVTQFa5do/edit?usp=drive_link&amp;ouid=105142876406402750370&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>Microareas Urbanas Parroquia Jose Vidal Marcano</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/presentation/d/1KXq6Ft8_zjFtJFWTyQJ9En7sti9Me7FB/edit?usp=drive_link&amp;ouid=105142876406402750370&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>Microareas Urbanas Parroquia Leonardo Ruiz Pineda</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/presentation/d/1BD6jFc7xyzviLIHrPbyIlcOU0UmUkX_9/edit?usp=drive_link&amp;ouid=105142876406402750370&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>Microareas Urbanas Parroquia Antonio José de Sucre</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/presentation/d/18XpV10Oke5oqgMfcjGxDfWOJ7itYllq_/edit?usp=drive_link&amp;ouid=105142876406402750370&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>Microareas Urbanas Parroquia San Rafael</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/presentation/d/1KS882cTzSaVGEAL6dEmcqg1mpQrPy6RH/edit?usp=drive_link&amp;ouid=105142876406402750370&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>Microareas Urbanas Parroquia San José</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/presentation/d/1P4-VJb-FPCIKC7rnon9N39oabgHC6ACI/edit?usp=drive_link&amp;ouid=105142876406402750370&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>Microareas Urbanas Parroquia Pedernales</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/presentation/d/15fXv89Yl0uNAGsm06xSx7aYjDCA4fcPl/edit?usp=drive_link&amp;ouid=105142876406402750370&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>PARROQUIA PEDERNALES</t>
+  </si>
+  <si>
+    <t>PARROQIUA LUIS BELTRAN PIETRO FIGUEROA</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/presentation/d/1oO5sIbje5OzQRle1UGJGjFzbHF1VqJUu/edit?usp=drive_link&amp;ouid=105142876406402750370&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>Microareas Urbanas Parroquia Luis Beltran Prieto Figueroa Capure</t>
   </si>
 </sst>
 </file>
@@ -1632,10 +1695,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J170"/>
+  <dimension ref="A1:J180"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="1" max="1" width="33.5703125" customWidth="1"/>
     <col min="2" max="2" width="21.140625" customWidth="1"/>
     <col min="3" max="3" width="59.28515625" customWidth="1"/>
     <col min="4" max="4" width="77.85546875" customWidth="1"/>
@@ -5259,7 +5322,225 @@
         <v>380</v>
       </c>
     </row>
+    <row r="171" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
+        <v>22</v>
+      </c>
+      <c r="B171" s="4">
+        <f t="shared" ref="B171" si="109">ROW(A170)</f>
+        <v>170</v>
+      </c>
+      <c r="C171" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="D171" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="E171" t="s">
+        <v>27</v>
+      </c>
+      <c r="F171" s="1" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="172" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
+        <v>24</v>
+      </c>
+      <c r="B172" s="4">
+        <f t="shared" ref="B172" si="110">ROW(A171)</f>
+        <v>171</v>
+      </c>
+      <c r="C172" s="5" t="s">
+        <v>384</v>
+      </c>
+      <c r="D172" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="E172" t="s">
+        <v>27</v>
+      </c>
+      <c r="F172" s="1" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
+        <v>18</v>
+      </c>
+      <c r="B173" s="4">
+        <f t="shared" ref="B173" si="111">ROW(A172)</f>
+        <v>172</v>
+      </c>
+      <c r="C173" s="5" t="s">
+        <v>386</v>
+      </c>
+      <c r="D173" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="E173" t="s">
+        <v>27</v>
+      </c>
+      <c r="F173" s="1" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="174" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
+        <v>22</v>
+      </c>
+      <c r="B174" s="4">
+        <f t="shared" ref="B174" si="112">ROW(A173)</f>
+        <v>173</v>
+      </c>
+      <c r="C174" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="D174" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="E174" t="s">
+        <v>27</v>
+      </c>
+      <c r="F174" s="1" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="175" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
+        <v>20</v>
+      </c>
+      <c r="B175" s="4">
+        <f t="shared" ref="B175" si="113">ROW(A174)</f>
+        <v>174</v>
+      </c>
+      <c r="C175" s="5" t="s">
+        <v>388</v>
+      </c>
+      <c r="D175" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="E175" t="s">
+        <v>27</v>
+      </c>
+      <c r="F175" s="1" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="176" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
+        <v>21</v>
+      </c>
+      <c r="B176" s="4">
+        <f t="shared" ref="B176" si="114">ROW(A175)</f>
+        <v>175</v>
+      </c>
+      <c r="C176" s="5" t="s">
+        <v>390</v>
+      </c>
+      <c r="D176" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="E176" t="s">
+        <v>27</v>
+      </c>
+      <c r="F176" s="1" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="177" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
+        <v>23</v>
+      </c>
+      <c r="B177" s="4">
+        <f t="shared" ref="B177" si="115">ROW(A176)</f>
+        <v>176</v>
+      </c>
+      <c r="C177" s="5" t="s">
+        <v>392</v>
+      </c>
+      <c r="D177" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="E177" t="s">
+        <v>27</v>
+      </c>
+      <c r="F177" s="1" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="178" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>17</v>
+      </c>
+      <c r="B178" s="4">
+        <f t="shared" ref="B178" si="116">ROW(A177)</f>
+        <v>177</v>
+      </c>
+      <c r="C178" s="5" t="s">
+        <v>394</v>
+      </c>
+      <c r="D178" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="E178" t="s">
+        <v>27</v>
+      </c>
+      <c r="F178" s="1" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="179" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>398</v>
+      </c>
+      <c r="B179" s="4">
+        <f t="shared" ref="B179" si="117">ROW(A178)</f>
+        <v>178</v>
+      </c>
+      <c r="C179" s="5" t="s">
+        <v>396</v>
+      </c>
+      <c r="D179" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="E179" t="s">
+        <v>27</v>
+      </c>
+      <c r="F179" s="1" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="180" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>399</v>
+      </c>
+      <c r="B180" s="4">
+        <f t="shared" ref="B180" si="118">ROW(A179)</f>
+        <v>179</v>
+      </c>
+      <c r="C180" s="5" t="s">
+        <v>401</v>
+      </c>
+      <c r="D180" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="E180" t="s">
+        <v>27</v>
+      </c>
+      <c r="F180" s="1" t="s">
+        <v>400</v>
+      </c>
+    </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Código de la dpt de parroquia" prompt="Código de la dpt de parroquia" sqref="A1">
+      <formula1>$A$2:$A$25</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A152:A178">
+      <formula1>$B$2:$B$25</formula1>
+    </dataValidation>
+  </dataValidations>
   <hyperlinks>
     <hyperlink ref="F26" r:id="rId1"/>
   </hyperlinks>
@@ -5273,27 +5554,27 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Código de la dpt de parroquia">
           <x14:formula1>
-            <xm:f>dpt_delta!$A$2:$A$24</xm:f>
+            <xm:f>dpt_delta!$A$2:$A$26</xm:f>
           </x14:formula1>
           <xm:sqref>A138:A151</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Código de la dpt de parroquia" prompt="Código de la dpt de parroquia">
           <x14:formula1>
-            <xm:f>dpt_delta!$A$2:$A$24</xm:f>
+            <xm:f>dpt_delta!$A$2:$A$26</xm:f>
           </x14:formula1>
-          <xm:sqref>A136:A137 A1</xm:sqref>
+          <xm:sqref>A136:A137</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>dpt_delta!$B$2:$B$24</xm:f>
+            <xm:f>dpt_delta!$B$2:$B$26</xm:f>
           </x14:formula1>
-          <xm:sqref>A2:A135 A152:A170</xm:sqref>
+          <xm:sqref>A2:A135 A180 A179</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Formato de la Publicación" prompt="Formato de la Publicación">
           <x14:formula1>
             <xm:f>formato!$A$2:$A$12</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E135 E152:E170</xm:sqref>
+          <xm:sqref>E2:E135 E152:E180</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -5330,10 +5611,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="38.7109375" customWidth="1"/>
+    <col min="2" max="2" width="41.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -5458,73 +5739,89 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>100400</v>
+        <v>100301</v>
       </c>
       <c r="B16" t="s">
-        <v>16</v>
+        <v>398</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>100401</v>
+        <v>100302</v>
       </c>
       <c r="B17" t="s">
-        <v>17</v>
+        <v>399</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>100402</v>
+        <v>100400</v>
       </c>
       <c r="B18" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>100403</v>
+        <v>100401</v>
       </c>
       <c r="B19" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>100404</v>
+        <v>100402</v>
       </c>
       <c r="B20" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>100405</v>
+        <v>100403</v>
       </c>
       <c r="B21" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>100406</v>
+        <v>100404</v>
       </c>
       <c r="B22" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>100407</v>
+        <v>100405</v>
       </c>
       <c r="B23" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
+        <v>100406</v>
+      </c>
+      <c r="B24" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>100407</v>
+      </c>
+      <c r="B25" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26">
         <v>100408</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B26" t="s">
         <v>24</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Se agregó las conunidades rurales de pedernales
</commit_message>
<xml_diff>
--- a/libro_publicaciones.xlsx
+++ b/libro_publicaciones.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="945" uniqueCount="402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="950" uniqueCount="405">
   <si>
     <t>codigo</t>
   </si>
@@ -1233,6 +1233,15 @@
   </si>
   <si>
     <t>Microareas Urbanas Parroquia Luis Beltran Prieto Figueroa Capure</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  PARROQUIA PEDERNALES</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CROQUIS DE LAS COMUNIDADES INDIGENA  PARROQUIA LUIS BELTRAN</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/presentation/d/1T8oQVk6AkToRhSfyRNn-Zoc4yJwX3AXK/edit?usp=drive_link&amp;ouid=105142876406402750370&amp;rtpof=true&amp;sd=true</t>
   </si>
 </sst>
 </file>
@@ -1695,7 +1704,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J180"/>
+  <dimension ref="A1:J181"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.5703125" customWidth="1"/>
@@ -5387,14 +5396,13 @@
     </row>
     <row r="174" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B174" s="4">
-        <f t="shared" ref="B174" si="112">ROW(A173)</f>
         <v>173</v>
       </c>
       <c r="C174" s="5" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="D174" s="5" t="s">
         <v>382</v>
@@ -5403,19 +5411,19 @@
         <v>27</v>
       </c>
       <c r="F174" s="1" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
     </row>
     <row r="175" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B175" s="4">
-        <f t="shared" ref="B175" si="113">ROW(A174)</f>
+        <f t="shared" ref="B175" si="112">ROW(A174)</f>
         <v>174</v>
       </c>
       <c r="C175" s="5" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="D175" s="5" t="s">
         <v>382</v>
@@ -5424,19 +5432,19 @@
         <v>27</v>
       </c>
       <c r="F175" s="1" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="176" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B176" s="4">
-        <f t="shared" ref="B176" si="114">ROW(A175)</f>
+        <f t="shared" ref="B176" si="113">ROW(A175)</f>
         <v>175</v>
       </c>
       <c r="C176" s="5" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="D176" s="5" t="s">
         <v>382</v>
@@ -5445,19 +5453,19 @@
         <v>27</v>
       </c>
       <c r="F176" s="1" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="177" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B177" s="4">
-        <f t="shared" ref="B177" si="115">ROW(A176)</f>
+        <f t="shared" ref="B177" si="114">ROW(A176)</f>
         <v>176</v>
       </c>
       <c r="C177" s="5" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="D177" s="5" t="s">
         <v>382</v>
@@ -5466,19 +5474,19 @@
         <v>27</v>
       </c>
       <c r="F177" s="1" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
     </row>
     <row r="178" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>17</v>
+        <v>398</v>
       </c>
       <c r="B178" s="4">
-        <f t="shared" ref="B178" si="116">ROW(A177)</f>
+        <f t="shared" ref="B178" si="115">ROW(A177)</f>
         <v>177</v>
       </c>
       <c r="C178" s="5" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D178" s="5" t="s">
         <v>382</v>
@@ -5487,19 +5495,19 @@
         <v>27</v>
       </c>
       <c r="F178" s="1" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
     </row>
     <row r="179" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B179" s="4">
-        <f t="shared" ref="B179" si="117">ROW(A178)</f>
+        <f t="shared" ref="B179" si="116">ROW(A178)</f>
         <v>178</v>
       </c>
       <c r="C179" s="5" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
       <c r="D179" s="5" t="s">
         <v>382</v>
@@ -5508,28 +5516,49 @@
         <v>27</v>
       </c>
       <c r="F179" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
     <row r="180" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B180" s="4">
-        <f t="shared" ref="B180" si="118">ROW(A179)</f>
+        <f t="shared" ref="B180" si="117">ROW(A179)</f>
         <v>179</v>
       </c>
       <c r="C180" s="5" t="s">
-        <v>401</v>
+        <v>55</v>
       </c>
       <c r="D180" s="5" t="s">
-        <v>382</v>
+        <v>402</v>
       </c>
       <c r="E180" t="s">
         <v>27</v>
       </c>
       <c r="F180" s="1" t="s">
-        <v>400</v>
+        <v>397</v>
+      </c>
+    </row>
+    <row r="181" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>399</v>
+      </c>
+      <c r="B181" s="4">
+        <f t="shared" ref="B181" si="118">ROW(A180)</f>
+        <v>180</v>
+      </c>
+      <c r="C181" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D181" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="E181" t="s">
+        <v>27</v>
+      </c>
+      <c r="F181" s="1" t="s">
+        <v>404</v>
       </c>
     </row>
   </sheetData>
@@ -5537,7 +5566,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Código de la dpt de parroquia" prompt="Código de la dpt de parroquia" sqref="A1">
       <formula1>$A$2:$A$25</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A152:A178">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A152:A177">
       <formula1>$B$2:$B$25</formula1>
     </dataValidation>
   </dataValidations>
@@ -5568,13 +5597,13 @@
           <x14:formula1>
             <xm:f>dpt_delta!$B$2:$B$26</xm:f>
           </x14:formula1>
-          <xm:sqref>A2:A135 A180 A179</xm:sqref>
+          <xm:sqref>A2:A135 A178:A181</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Formato de la Publicación" prompt="Formato de la Publicación">
           <x14:formula1>
             <xm:f>formato!$A$2:$A$12</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E135 E152:E180</xm:sqref>
+          <xm:sqref>E2:E135 E152:E181</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Se Modificó la parroquia pedernales
</commit_message>
<xml_diff>
--- a/libro_publicaciones.xlsx
+++ b/libro_publicaciones.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="950" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="950" uniqueCount="406">
   <si>
     <t>codigo</t>
   </si>
@@ -1242,6 +1242,9 @@
   </si>
   <si>
     <t>https://docs.google.com/presentation/d/1T8oQVk6AkToRhSfyRNn-Zoc4yJwX3AXK/edit?usp=drive_link&amp;ouid=105142876406402750370&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/presentation/d/1ftpq1QunglQuiNZKBNZMD9MIcWZuH0P0/edit?usp=drive_link&amp;ouid=105142876406402750370&amp;rtpof=true&amp;sd=true</t>
   </si>
 </sst>
 </file>
@@ -1707,7 +1710,7 @@
   <dimension ref="A1:J181"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33.5703125" customWidth="1"/>
+    <col min="1" max="1" width="44.5703125" customWidth="1"/>
     <col min="2" max="2" width="21.140625" customWidth="1"/>
     <col min="3" max="3" width="59.28515625" customWidth="1"/>
     <col min="4" max="4" width="77.85546875" customWidth="1"/>
@@ -5537,7 +5540,7 @@
         <v>27</v>
       </c>
       <c r="F180" s="1" t="s">
-        <v>397</v>
+        <v>405</v>
       </c>
     </row>
     <row r="181" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>